<commit_message>
Add .gitattributes for consistent line endings across machines
</commit_message>
<xml_diff>
--- a/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
+++ b/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6310" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6310"/>
   </bookViews>
   <sheets>
     <sheet name="tabla x hora" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="67">
   <si>
     <t>Florida</t>
   </si>
@@ -224,6 +224,15 @@
   </si>
   <si>
     <t>Nueva_tienda</t>
+  </si>
+  <si>
+    <t>Ariganello Melina</t>
+  </si>
+  <si>
+    <t>Hernandez Guerrero Helen Siloe</t>
+  </si>
+  <si>
+    <t>Nayla Rotela</t>
   </si>
 </sst>
 </file>
@@ -1939,7 +1948,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P233"/>
+  <dimension ref="A1:P260"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.54296875" style="4"/>
@@ -5373,7 +5382,7 @@
         <v>75</v>
       </c>
       <c r="N173" s="4">
-        <f t="shared" ref="N173:N233" si="3">SUM(D173:M173)</f>
+        <f t="shared" ref="N173:N235" si="3">SUM(D173:M173)</f>
         <v>75</v>
       </c>
     </row>
@@ -6509,6 +6518,528 @@
       <c r="N233" s="4">
         <f t="shared" si="3"/>
         <v>13</v>
+      </c>
+    </row>
+    <row r="234" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A234" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B234" s="4">
+        <v>3</v>
+      </c>
+      <c r="C234" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D234" s="4">
+        <v>75</v>
+      </c>
+      <c r="H234" s="4">
+        <v>45</v>
+      </c>
+      <c r="N234" s="4">
+        <f t="shared" si="3"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="235" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A235" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B235" s="4">
+        <v>4</v>
+      </c>
+      <c r="C235" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D235" s="5">
+        <v>126</v>
+      </c>
+      <c r="N235" s="4">
+        <f t="shared" si="3"/>
+        <v>126</v>
+      </c>
+    </row>
+    <row r="236" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A236" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B236" s="4">
+        <v>10</v>
+      </c>
+      <c r="C236" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L236" s="4">
+        <v>104</v>
+      </c>
+      <c r="N236" s="4">
+        <f t="shared" ref="N236:N260" si="4">SUM(D236:M236)</f>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="237" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A237" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B237" s="4">
+        <v>11</v>
+      </c>
+      <c r="C237" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I237" s="4">
+        <v>112</v>
+      </c>
+      <c r="N237" s="4">
+        <f t="shared" si="4"/>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="238" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A238" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B238" s="4">
+        <v>12</v>
+      </c>
+      <c r="C238" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H238" s="4">
+        <v>69</v>
+      </c>
+      <c r="N238" s="4">
+        <f t="shared" si="4"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="239" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A239" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B239" s="4">
+        <v>14</v>
+      </c>
+      <c r="C239" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I239" s="4">
+        <v>107</v>
+      </c>
+      <c r="N239" s="4">
+        <f t="shared" si="4"/>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="240" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A240" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B240" s="4">
+        <v>15</v>
+      </c>
+      <c r="C240" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L240" s="4">
+        <v>100</v>
+      </c>
+      <c r="N240" s="4">
+        <f t="shared" si="4"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="241" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A241" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B241" s="4">
+        <v>18</v>
+      </c>
+      <c r="C241" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D241" s="4">
+        <v>12</v>
+      </c>
+      <c r="E241" s="5">
+        <v>99</v>
+      </c>
+      <c r="H241" s="4">
+        <v>21</v>
+      </c>
+      <c r="N241" s="4">
+        <f t="shared" si="4"/>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="242" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A242" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B242" s="4">
+        <v>19</v>
+      </c>
+      <c r="C242" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E242" s="4">
+        <v>132</v>
+      </c>
+      <c r="N242" s="4">
+        <f t="shared" si="4"/>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="243" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A243" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B243" s="4">
+        <v>20</v>
+      </c>
+      <c r="C243" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H243" s="4">
+        <v>132</v>
+      </c>
+      <c r="N243" s="4">
+        <f t="shared" si="4"/>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="244" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A244" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B244" s="4">
+        <v>27</v>
+      </c>
+      <c r="C244" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K244" s="4">
+        <v>113</v>
+      </c>
+      <c r="N244" s="4">
+        <f t="shared" si="4"/>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="245" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A245" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B245" s="4">
+        <v>28</v>
+      </c>
+      <c r="C245" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K245" s="4">
+        <v>113</v>
+      </c>
+      <c r="N245" s="4">
+        <f t="shared" si="4"/>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="246" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A246" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B246" s="4">
+        <v>29</v>
+      </c>
+      <c r="C246" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J246" s="4">
+        <v>63</v>
+      </c>
+      <c r="K246" s="4">
+        <v>49</v>
+      </c>
+      <c r="N246" s="4">
+        <f t="shared" si="4"/>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="247" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A247" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B247" s="4">
+        <v>31</v>
+      </c>
+      <c r="C247" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J247" s="4">
+        <v>110</v>
+      </c>
+      <c r="N247" s="4">
+        <f t="shared" si="4"/>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="248" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A248" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B248" s="4">
+        <v>36</v>
+      </c>
+      <c r="C248" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F248" s="4">
+        <v>68</v>
+      </c>
+      <c r="M248" s="4">
+        <v>55</v>
+      </c>
+      <c r="N248" s="4">
+        <f t="shared" si="4"/>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="249" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A249" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B249" s="4">
+        <v>39</v>
+      </c>
+      <c r="C249" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I249" s="4">
+        <v>94</v>
+      </c>
+      <c r="K249" s="5">
+        <v>12</v>
+      </c>
+      <c r="N249" s="4">
+        <f t="shared" si="4"/>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="250" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A250" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B250" s="4">
+        <v>41</v>
+      </c>
+      <c r="C250" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F250" s="4">
+        <v>9</v>
+      </c>
+      <c r="M250" s="4">
+        <v>113</v>
+      </c>
+      <c r="N250" s="4">
+        <f t="shared" si="4"/>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="251" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A251" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B251" s="4">
+        <v>42</v>
+      </c>
+      <c r="C251" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D251" s="4">
+        <v>125</v>
+      </c>
+      <c r="N251" s="4">
+        <f t="shared" si="4"/>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="252" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A252" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B252" s="4">
+        <v>44</v>
+      </c>
+      <c r="C252" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D252" s="4">
+        <v>20</v>
+      </c>
+      <c r="N252" s="4">
+        <f t="shared" si="4"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="253" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A253" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B253" s="4">
+        <v>47</v>
+      </c>
+      <c r="C253" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D253" s="4">
+        <v>49</v>
+      </c>
+      <c r="H253" s="4">
+        <v>69</v>
+      </c>
+      <c r="N253" s="4">
+        <f t="shared" si="4"/>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="254" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A254" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B254" s="4">
+        <v>49</v>
+      </c>
+      <c r="C254" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J254" s="4">
+        <v>102</v>
+      </c>
+      <c r="N254" s="4">
+        <f t="shared" si="4"/>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="255" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A255" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B255" s="4">
+        <v>52</v>
+      </c>
+      <c r="C255" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="L255" s="4">
+        <v>89</v>
+      </c>
+      <c r="N255" s="4">
+        <f t="shared" si="4"/>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="256" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A256" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B256" s="4">
+        <v>54</v>
+      </c>
+      <c r="C256" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E256" s="4">
+        <v>18</v>
+      </c>
+      <c r="F256" s="4">
+        <v>87</v>
+      </c>
+      <c r="M256" s="4">
+        <v>12</v>
+      </c>
+      <c r="N256" s="4">
+        <f t="shared" si="4"/>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="257" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A257" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B257" s="4">
+        <v>58</v>
+      </c>
+      <c r="C257" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D257" s="4">
+        <v>115</v>
+      </c>
+      <c r="N257" s="4">
+        <f t="shared" si="4"/>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="258" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A258" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B258" s="4">
+        <v>59</v>
+      </c>
+      <c r="C258" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F258" s="4">
+        <v>16</v>
+      </c>
+      <c r="M258" s="4">
+        <v>61</v>
+      </c>
+      <c r="N258" s="4">
+        <f t="shared" si="4"/>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="259" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A259" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B259" s="4">
+        <v>60</v>
+      </c>
+      <c r="C259" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F259" s="4">
+        <v>17</v>
+      </c>
+      <c r="M259" s="4">
+        <v>65</v>
+      </c>
+      <c r="N259" s="4">
+        <f t="shared" si="4"/>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="260" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A260" s="3">
+        <v>46143</v>
+      </c>
+      <c r="B260" s="4">
+        <v>61</v>
+      </c>
+      <c r="C260" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D260" s="4">
+        <v>53</v>
+      </c>
+      <c r="N260" s="4">
+        <f t="shared" si="4"/>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -6726,6 +7257,13 @@
       <c r="C17" t="s">
         <v>2</v>
       </c>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10">
+        <v>46143</v>
+      </c>
+      <c r="F17" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
@@ -6889,6 +7427,9 @@
       <c r="C29" t="s">
         <v>0</v>
       </c>
+      <c r="D29" s="10">
+        <v>46149</v>
+      </c>
       <c r="E29" s="10">
         <v>46113</v>
       </c>
@@ -6933,6 +7474,9 @@
       </c>
       <c r="C32" t="s">
         <v>0</v>
+      </c>
+      <c r="D32" s="10">
+        <v>46171</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Add .gitattributes to manage line endings
</commit_message>
<xml_diff>
--- a/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
+++ b/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maval\Documents\Vale laburo\Castelli\Reportes\Reporte_gastos\Sueldos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Valeria\Reportes\Reporte_gastos\Sueldos\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tabla x hora'!$A$1:$O$233</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tabla x hora'!$A$1:$O$260</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'vendedora-tienda'!$A$1:$F$37</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -6683,12 +6683,12 @@
       <c r="C242" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E242" s="4">
-        <v>132</v>
+      <c r="M242" s="4">
+        <v>124</v>
       </c>
       <c r="N242" s="4">
         <f t="shared" si="4"/>
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="243" spans="1:14" x14ac:dyDescent="0.35">
@@ -7043,7 +7043,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O233"/>
+  <autoFilter ref="A1:O260"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
sigo trabajando en gastos y sueldos
</commit_message>
<xml_diff>
--- a/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
+++ b/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maval\Documents\Vale laburo\Castelli\Reportes\Reporte_gastos\Sueldos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Valeria\Reportes\Reporte_gastos\Sueldos\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6312"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6310"/>
   </bookViews>
   <sheets>
     <sheet name="tabla x hora" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="71">
   <si>
     <t>Florida</t>
   </si>
@@ -243,6 +243,9 @@
   <si>
     <t>Vacaciones</t>
   </si>
+  <si>
+    <t>son 14 días de vacaciones según el recibo. En archivo horas figuran 11</t>
+  </si>
 </sst>
 </file>
 
@@ -425,7 +428,9 @@
           <cell r="B2" t="str">
             <v>Viña Sofia</v>
           </cell>
-          <cell r="C2"/>
+          <cell r="C2">
+            <v>0</v>
+          </cell>
           <cell r="D2" t="str">
             <v>LU Florida</v>
           </cell>
@@ -438,12 +443,18 @@
           <cell r="G2">
             <v>5</v>
           </cell>
-          <cell r="H2"/>
-          <cell r="I2"/>
+          <cell r="H2">
+            <v>0</v>
+          </cell>
+          <cell r="I2">
+            <v>0</v>
+          </cell>
           <cell r="J2" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K2"/>
+          <cell r="K2">
+            <v>0</v>
+          </cell>
           <cell r="L2">
             <v>58953</v>
           </cell>
@@ -470,23 +481,33 @@
           <cell r="B3" t="str">
             <v>Urbieta Barbara Giselle</v>
           </cell>
-          <cell r="C3"/>
+          <cell r="C3">
+            <v>0</v>
+          </cell>
           <cell r="D3" t="str">
             <v>LU Florida</v>
           </cell>
           <cell r="E3">
             <v>8</v>
           </cell>
-          <cell r="F3"/>
+          <cell r="F3">
+            <v>0</v>
+          </cell>
           <cell r="G3">
             <v>8</v>
           </cell>
-          <cell r="H3"/>
-          <cell r="I3"/>
+          <cell r="H3">
+            <v>0</v>
+          </cell>
+          <cell r="I3">
+            <v>0</v>
+          </cell>
           <cell r="J3" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K3"/>
+          <cell r="K3">
+            <v>0</v>
+          </cell>
           <cell r="L3">
             <v>0</v>
           </cell>
@@ -502,7 +523,9 @@
           <cell r="P3">
             <v>1557231.8177199899</v>
           </cell>
-          <cell r="Q3"/>
+          <cell r="Q3">
+            <v>0</v>
+          </cell>
         </row>
         <row r="4">
           <cell r="A4">
@@ -511,7 +534,9 @@
           <cell r="B4" t="str">
             <v>Ruiz de la Torre Maitena</v>
           </cell>
-          <cell r="C4"/>
+          <cell r="C4">
+            <v>0</v>
+          </cell>
           <cell r="D4" t="str">
             <v>LU Florida</v>
           </cell>
@@ -524,12 +549,18 @@
           <cell r="G4">
             <v>5</v>
           </cell>
-          <cell r="H4"/>
-          <cell r="I4"/>
+          <cell r="H4">
+            <v>0</v>
+          </cell>
+          <cell r="I4">
+            <v>0</v>
+          </cell>
           <cell r="J4" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K4"/>
+          <cell r="K4">
+            <v>0</v>
+          </cell>
           <cell r="L4">
             <v>58904</v>
           </cell>
@@ -556,7 +587,9 @@
           <cell r="B5" t="str">
             <v>Imperiale Candela</v>
           </cell>
-          <cell r="C5"/>
+          <cell r="C5">
+            <v>0</v>
+          </cell>
           <cell r="D5" t="str">
             <v>LU Florida</v>
           </cell>
@@ -569,12 +602,18 @@
           <cell r="G5">
             <v>5</v>
           </cell>
-          <cell r="H5"/>
-          <cell r="I5"/>
+          <cell r="H5">
+            <v>0</v>
+          </cell>
+          <cell r="I5">
+            <v>0</v>
+          </cell>
           <cell r="J5" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K5"/>
+          <cell r="K5">
+            <v>0</v>
+          </cell>
           <cell r="L5">
             <v>65164</v>
           </cell>
@@ -601,21 +640,33 @@
           <cell r="B6" t="str">
             <v>Balmaceda Luciana</v>
           </cell>
-          <cell r="C6"/>
+          <cell r="C6">
+            <v>0</v>
+          </cell>
           <cell r="D6" t="str">
             <v>LU Florida</v>
           </cell>
           <cell r="E6">
             <v>0</v>
           </cell>
-          <cell r="F6"/>
-          <cell r="G6"/>
-          <cell r="H6"/>
-          <cell r="I6"/>
+          <cell r="F6">
+            <v>0</v>
+          </cell>
+          <cell r="G6">
+            <v>0</v>
+          </cell>
+          <cell r="H6">
+            <v>0</v>
+          </cell>
+          <cell r="I6">
+            <v>0</v>
+          </cell>
           <cell r="J6" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K6"/>
+          <cell r="K6">
+            <v>0</v>
+          </cell>
           <cell r="L6">
             <v>0</v>
           </cell>
@@ -631,7 +682,9 @@
           <cell r="P6">
             <v>1355</v>
           </cell>
-          <cell r="Q6"/>
+          <cell r="Q6">
+            <v>0</v>
+          </cell>
         </row>
         <row r="7">
           <cell r="A7">
@@ -640,23 +693,33 @@
           <cell r="B7" t="str">
             <v>Cabovianco Natalia</v>
           </cell>
-          <cell r="C7"/>
+          <cell r="C7">
+            <v>0</v>
+          </cell>
           <cell r="D7" t="str">
             <v>AS San Telmo</v>
           </cell>
           <cell r="E7">
             <v>8</v>
           </cell>
-          <cell r="F7"/>
+          <cell r="F7">
+            <v>0</v>
+          </cell>
           <cell r="G7">
             <v>8</v>
           </cell>
-          <cell r="H7"/>
-          <cell r="I7"/>
+          <cell r="H7">
+            <v>0</v>
+          </cell>
+          <cell r="I7">
+            <v>0</v>
+          </cell>
           <cell r="J7" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K7"/>
+          <cell r="K7">
+            <v>0</v>
+          </cell>
           <cell r="L7">
             <v>0</v>
           </cell>
@@ -672,7 +735,9 @@
           <cell r="P7">
             <v>1788196.15377499</v>
           </cell>
-          <cell r="Q7"/>
+          <cell r="Q7">
+            <v>0</v>
+          </cell>
         </row>
         <row r="8">
           <cell r="A8">
@@ -681,7 +746,9 @@
           <cell r="B8" t="str">
             <v>Carrizo Camila</v>
           </cell>
-          <cell r="C8"/>
+          <cell r="C8">
+            <v>0</v>
+          </cell>
           <cell r="D8" t="str">
             <v>AS San Telmo</v>
           </cell>
@@ -694,12 +761,18 @@
           <cell r="G8">
             <v>4</v>
           </cell>
-          <cell r="H8"/>
-          <cell r="I8"/>
+          <cell r="H8">
+            <v>0</v>
+          </cell>
+          <cell r="I8">
+            <v>0</v>
+          </cell>
           <cell r="J8" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K8"/>
+          <cell r="K8">
+            <v>0</v>
+          </cell>
           <cell r="L8">
             <v>33535</v>
           </cell>
@@ -726,7 +799,9 @@
           <cell r="B9" t="str">
             <v>Esposito Candela</v>
           </cell>
-          <cell r="C9"/>
+          <cell r="C9">
+            <v>0</v>
+          </cell>
           <cell r="D9" t="str">
             <v>Lucero ST1</v>
           </cell>
@@ -739,14 +814,18 @@
           <cell r="G9">
             <v>5</v>
           </cell>
-          <cell r="H9"/>
+          <cell r="H9">
+            <v>0</v>
+          </cell>
           <cell r="I9">
             <v>12</v>
           </cell>
           <cell r="J9" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K9"/>
+          <cell r="K9">
+            <v>0</v>
+          </cell>
           <cell r="L9">
             <v>59262</v>
           </cell>
@@ -773,7 +852,9 @@
           <cell r="B10" t="str">
             <v>Barajas Barbara</v>
           </cell>
-          <cell r="C10"/>
+          <cell r="C10">
+            <v>0</v>
+          </cell>
           <cell r="D10" t="str">
             <v>Recoleta</v>
           </cell>
@@ -786,12 +867,18 @@
           <cell r="G10">
             <v>6</v>
           </cell>
-          <cell r="H10"/>
-          <cell r="I10"/>
+          <cell r="H10">
+            <v>0</v>
+          </cell>
+          <cell r="I10">
+            <v>0</v>
+          </cell>
           <cell r="J10" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K10"/>
+          <cell r="K10">
+            <v>0</v>
+          </cell>
           <cell r="L10">
             <v>54186</v>
           </cell>
@@ -818,7 +905,9 @@
           <cell r="B11" t="str">
             <v>De Brito Rocio</v>
           </cell>
-          <cell r="C11"/>
+          <cell r="C11">
+            <v>0</v>
+          </cell>
           <cell r="D11" t="str">
             <v>Güemes</v>
           </cell>
@@ -828,13 +917,21 @@
           <cell r="F11" t="str">
             <v>125.00</v>
           </cell>
-          <cell r="G11"/>
-          <cell r="H11"/>
-          <cell r="I11"/>
+          <cell r="G11">
+            <v>0</v>
+          </cell>
+          <cell r="H11">
+            <v>0</v>
+          </cell>
+          <cell r="I11">
+            <v>0</v>
+          </cell>
           <cell r="J11" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K11"/>
+          <cell r="K11">
+            <v>0</v>
+          </cell>
           <cell r="L11">
             <v>9173</v>
           </cell>
@@ -861,7 +958,9 @@
           <cell r="B12" t="str">
             <v>Lara Robbio</v>
           </cell>
-          <cell r="C12"/>
+          <cell r="C12">
+            <v>0</v>
+          </cell>
           <cell r="D12" t="str">
             <v>Lucero ST1</v>
           </cell>
@@ -874,14 +973,18 @@
           <cell r="G12">
             <v>5</v>
           </cell>
-          <cell r="H12"/>
+          <cell r="H12">
+            <v>0</v>
+          </cell>
           <cell r="I12">
             <v>8</v>
           </cell>
           <cell r="J12" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K12"/>
+          <cell r="K12">
+            <v>0</v>
+          </cell>
           <cell r="L12">
             <v>62585</v>
           </cell>
@@ -908,7 +1011,9 @@
           <cell r="B13" t="str">
             <v>Molina Agustina</v>
           </cell>
-          <cell r="C13"/>
+          <cell r="C13">
+            <v>0</v>
+          </cell>
           <cell r="D13" t="str">
             <v>AS San Telmo</v>
           </cell>
@@ -921,12 +1026,18 @@
           <cell r="G13">
             <v>4</v>
           </cell>
-          <cell r="H13"/>
-          <cell r="I13"/>
+          <cell r="H13">
+            <v>0</v>
+          </cell>
+          <cell r="I13">
+            <v>0</v>
+          </cell>
           <cell r="J13" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K13"/>
+          <cell r="K13">
+            <v>0</v>
+          </cell>
           <cell r="L13">
             <v>32724</v>
           </cell>
@@ -953,7 +1064,9 @@
           <cell r="B14" t="str">
             <v>CORONEL Mailen</v>
           </cell>
-          <cell r="C14"/>
+          <cell r="C14">
+            <v>0</v>
+          </cell>
           <cell r="D14" t="str">
             <v>Güemes</v>
           </cell>
@@ -966,14 +1079,18 @@
           <cell r="G14">
             <v>5</v>
           </cell>
-          <cell r="H14"/>
+          <cell r="H14">
+            <v>0</v>
+          </cell>
           <cell r="I14">
             <v>8</v>
           </cell>
           <cell r="J14" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K14"/>
+          <cell r="K14">
+            <v>0</v>
+          </cell>
           <cell r="L14">
             <v>20449</v>
           </cell>
@@ -1000,7 +1117,9 @@
           <cell r="B15" t="str">
             <v>Gimenez Candela</v>
           </cell>
-          <cell r="C15"/>
+          <cell r="C15">
+            <v>0</v>
+          </cell>
           <cell r="D15" t="str">
             <v>Recoleta</v>
           </cell>
@@ -1010,13 +1129,21 @@
           <cell r="F15" t="str">
             <v>132.00</v>
           </cell>
-          <cell r="G15"/>
-          <cell r="H15"/>
-          <cell r="I15"/>
+          <cell r="G15">
+            <v>0</v>
+          </cell>
+          <cell r="H15">
+            <v>0</v>
+          </cell>
+          <cell r="I15">
+            <v>0</v>
+          </cell>
           <cell r="J15" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K15"/>
+          <cell r="K15">
+            <v>0</v>
+          </cell>
           <cell r="L15">
             <v>22621</v>
           </cell>
@@ -1043,7 +1170,9 @@
           <cell r="B16" t="str">
             <v>Oliva Micaela</v>
           </cell>
-          <cell r="C16"/>
+          <cell r="C16">
+            <v>0</v>
+          </cell>
           <cell r="D16" t="str">
             <v>Recoleta</v>
           </cell>
@@ -1056,12 +1185,18 @@
           <cell r="G16">
             <v>5</v>
           </cell>
-          <cell r="H16"/>
-          <cell r="I16"/>
+          <cell r="H16">
+            <v>0</v>
+          </cell>
+          <cell r="I16">
+            <v>0</v>
+          </cell>
           <cell r="J16" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K16"/>
+          <cell r="K16">
+            <v>0</v>
+          </cell>
           <cell r="L16">
             <v>54186</v>
           </cell>
@@ -1088,7 +1223,9 @@
           <cell r="B17" t="str">
             <v>Mohamad Daila</v>
           </cell>
-          <cell r="C17"/>
+          <cell r="C17">
+            <v>0</v>
+          </cell>
           <cell r="D17" t="str">
             <v>Lucero ST1</v>
           </cell>
@@ -1101,12 +1238,18 @@
           <cell r="G17">
             <v>4</v>
           </cell>
-          <cell r="H17"/>
-          <cell r="I17"/>
+          <cell r="H17">
+            <v>0</v>
+          </cell>
+          <cell r="I17">
+            <v>0</v>
+          </cell>
           <cell r="J17" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K17"/>
+          <cell r="K17">
+            <v>0</v>
+          </cell>
           <cell r="L17">
             <v>54835</v>
           </cell>
@@ -1133,7 +1276,9 @@
           <cell r="B18" t="str">
             <v>Bertolo Milagros</v>
           </cell>
-          <cell r="C18"/>
+          <cell r="C18">
+            <v>0</v>
+          </cell>
           <cell r="D18" t="str">
             <v>French</v>
           </cell>
@@ -1143,13 +1288,21 @@
           <cell r="F18">
             <v>115</v>
           </cell>
-          <cell r="G18"/>
-          <cell r="H18"/>
-          <cell r="I18"/>
+          <cell r="G18">
+            <v>0</v>
+          </cell>
+          <cell r="H18">
+            <v>0</v>
+          </cell>
+          <cell r="I18">
+            <v>0</v>
+          </cell>
           <cell r="J18" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K18"/>
+          <cell r="K18">
+            <v>0</v>
+          </cell>
           <cell r="L18">
             <v>47914</v>
           </cell>
@@ -1176,7 +1329,9 @@
           <cell r="B19" t="str">
             <v>Machuca Araceli</v>
           </cell>
-          <cell r="C19"/>
+          <cell r="C19">
+            <v>0</v>
+          </cell>
           <cell r="D19" t="str">
             <v>French</v>
           </cell>
@@ -1189,12 +1344,18 @@
           <cell r="G19" t="str">
             <v>4.00</v>
           </cell>
-          <cell r="H19"/>
-          <cell r="I19"/>
+          <cell r="H19">
+            <v>0</v>
+          </cell>
+          <cell r="I19">
+            <v>0</v>
+          </cell>
           <cell r="J19" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K19"/>
+          <cell r="K19">
+            <v>0</v>
+          </cell>
           <cell r="L19">
             <v>38788</v>
           </cell>
@@ -1221,7 +1382,9 @@
           <cell r="B20" t="str">
             <v>Scholler Chavez Ruth</v>
           </cell>
-          <cell r="C20"/>
+          <cell r="C20">
+            <v>0</v>
+          </cell>
           <cell r="D20" t="str">
             <v>French</v>
           </cell>
@@ -1234,12 +1397,18 @@
           <cell r="G20" t="str">
             <v>4.00</v>
           </cell>
-          <cell r="H20"/>
-          <cell r="I20"/>
+          <cell r="H20">
+            <v>0</v>
+          </cell>
+          <cell r="I20">
+            <v>0</v>
+          </cell>
           <cell r="J20" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K20"/>
+          <cell r="K20">
+            <v>0</v>
+          </cell>
           <cell r="L20">
             <v>38168</v>
           </cell>
@@ -1266,7 +1435,9 @@
           <cell r="B21" t="str">
             <v>Anabella Baragatti</v>
           </cell>
-          <cell r="C21"/>
+          <cell r="C21">
+            <v>0</v>
+          </cell>
           <cell r="D21" t="str">
             <v>LU Florida</v>
           </cell>
@@ -1279,12 +1450,18 @@
           <cell r="G21">
             <v>4</v>
           </cell>
-          <cell r="H21"/>
-          <cell r="I21"/>
+          <cell r="H21">
+            <v>0</v>
+          </cell>
+          <cell r="I21">
+            <v>0</v>
+          </cell>
           <cell r="J21" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K21"/>
+          <cell r="K21">
+            <v>0</v>
+          </cell>
           <cell r="L21">
             <v>0</v>
           </cell>
@@ -1311,7 +1488,9 @@
           <cell r="B22" t="str">
             <v>Gisela Bonino</v>
           </cell>
-          <cell r="C22"/>
+          <cell r="C22">
+            <v>0</v>
+          </cell>
           <cell r="D22" t="str">
             <v>Lucero ST2</v>
           </cell>
@@ -1324,12 +1503,18 @@
           <cell r="G22">
             <v>5</v>
           </cell>
-          <cell r="H22"/>
-          <cell r="I22"/>
+          <cell r="H22">
+            <v>0</v>
+          </cell>
+          <cell r="I22">
+            <v>0</v>
+          </cell>
           <cell r="J22" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K22"/>
+          <cell r="K22">
+            <v>0</v>
+          </cell>
           <cell r="L22">
             <v>0</v>
           </cell>
@@ -1356,7 +1541,9 @@
           <cell r="B23" t="str">
             <v>Dana Ramirez</v>
           </cell>
-          <cell r="C23"/>
+          <cell r="C23">
+            <v>0</v>
+          </cell>
           <cell r="D23" t="str">
             <v>AS San Telmo</v>
           </cell>
@@ -1369,12 +1556,18 @@
           <cell r="G23">
             <v>4</v>
           </cell>
-          <cell r="H23"/>
-          <cell r="I23"/>
+          <cell r="H23">
+            <v>0</v>
+          </cell>
+          <cell r="I23">
+            <v>0</v>
+          </cell>
           <cell r="J23" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K23"/>
+          <cell r="K23">
+            <v>0</v>
+          </cell>
           <cell r="L23">
             <v>0</v>
           </cell>
@@ -1401,7 +1594,9 @@
           <cell r="B24" t="str">
             <v>Diaz Dulcinea</v>
           </cell>
-          <cell r="C24"/>
+          <cell r="C24">
+            <v>0</v>
+          </cell>
           <cell r="D24" t="str">
             <v>LU Florida</v>
           </cell>
@@ -1411,13 +1606,21 @@
           <cell r="F24">
             <v>117</v>
           </cell>
-          <cell r="G24"/>
-          <cell r="H24"/>
-          <cell r="I24"/>
+          <cell r="G24">
+            <v>0</v>
+          </cell>
+          <cell r="H24">
+            <v>0</v>
+          </cell>
+          <cell r="I24">
+            <v>0</v>
+          </cell>
           <cell r="J24" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K24"/>
+          <cell r="K24">
+            <v>0</v>
+          </cell>
           <cell r="L24">
             <v>0</v>
           </cell>
@@ -1444,7 +1647,9 @@
           <cell r="B25" t="str">
             <v>Schiavone Fiona Ludmila</v>
           </cell>
-          <cell r="C25"/>
+          <cell r="C25">
+            <v>0</v>
+          </cell>
           <cell r="D25" t="str">
             <v>El Solar</v>
           </cell>
@@ -1454,13 +1659,21 @@
           <cell r="F25" t="str">
             <v>89.00</v>
           </cell>
-          <cell r="G25"/>
-          <cell r="H25"/>
-          <cell r="I25"/>
+          <cell r="G25">
+            <v>0</v>
+          </cell>
+          <cell r="H25">
+            <v>0</v>
+          </cell>
+          <cell r="I25">
+            <v>0</v>
+          </cell>
           <cell r="J25" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K25"/>
+          <cell r="K25">
+            <v>0</v>
+          </cell>
           <cell r="L25">
             <v>0</v>
           </cell>
@@ -1487,7 +1700,9 @@
           <cell r="B26" t="str">
             <v>Perazzo Juana</v>
           </cell>
-          <cell r="C26"/>
+          <cell r="C26">
+            <v>0</v>
+          </cell>
           <cell r="D26" t="str">
             <v>El Solar</v>
           </cell>
@@ -1497,13 +1712,21 @@
           <cell r="F26" t="str">
             <v>87.00</v>
           </cell>
-          <cell r="G26"/>
-          <cell r="H26"/>
-          <cell r="I26"/>
+          <cell r="G26">
+            <v>0</v>
+          </cell>
+          <cell r="H26">
+            <v>0</v>
+          </cell>
+          <cell r="I26">
+            <v>0</v>
+          </cell>
           <cell r="J26" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K26"/>
+          <cell r="K26">
+            <v>0</v>
+          </cell>
           <cell r="L26">
             <v>0</v>
           </cell>
@@ -1530,7 +1753,9 @@
           <cell r="B27" t="str">
             <v>Delgado Maria Paz</v>
           </cell>
-          <cell r="C27"/>
+          <cell r="C27">
+            <v>0</v>
+          </cell>
           <cell r="D27" t="str">
             <v>El Solar</v>
           </cell>
@@ -1540,13 +1765,21 @@
           <cell r="F27">
             <v>88</v>
           </cell>
-          <cell r="G27"/>
-          <cell r="H27"/>
-          <cell r="I27"/>
+          <cell r="G27">
+            <v>0</v>
+          </cell>
+          <cell r="H27">
+            <v>0</v>
+          </cell>
+          <cell r="I27">
+            <v>0</v>
+          </cell>
           <cell r="J27" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K27"/>
+          <cell r="K27">
+            <v>0</v>
+          </cell>
           <cell r="L27">
             <v>0</v>
           </cell>
@@ -1573,7 +1806,9 @@
           <cell r="B28" t="str">
             <v>Giordano Carolina Inez</v>
           </cell>
-          <cell r="C28"/>
+          <cell r="C28">
+            <v>0</v>
+          </cell>
           <cell r="D28" t="str">
             <v>Lucero ST 2</v>
           </cell>
@@ -1583,13 +1818,21 @@
           <cell r="F28">
             <v>67</v>
           </cell>
-          <cell r="G28"/>
-          <cell r="H28"/>
-          <cell r="I28"/>
+          <cell r="G28">
+            <v>0</v>
+          </cell>
+          <cell r="H28">
+            <v>0</v>
+          </cell>
+          <cell r="I28">
+            <v>0</v>
+          </cell>
           <cell r="J28" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K28"/>
+          <cell r="K28">
+            <v>0</v>
+          </cell>
           <cell r="L28">
             <v>0</v>
           </cell>
@@ -1616,7 +1859,9 @@
           <cell r="B29" t="str">
             <v>Martinez Franzi Lourdes</v>
           </cell>
-          <cell r="C29"/>
+          <cell r="C29">
+            <v>0</v>
+          </cell>
           <cell r="D29" t="str">
             <v>El Solar</v>
           </cell>
@@ -1626,13 +1871,21 @@
           <cell r="F29">
             <v>76</v>
           </cell>
-          <cell r="G29"/>
-          <cell r="H29"/>
-          <cell r="I29"/>
+          <cell r="G29">
+            <v>0</v>
+          </cell>
+          <cell r="H29">
+            <v>0</v>
+          </cell>
+          <cell r="I29">
+            <v>0</v>
+          </cell>
           <cell r="J29" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K29"/>
+          <cell r="K29">
+            <v>0</v>
+          </cell>
           <cell r="L29">
             <v>0</v>
           </cell>
@@ -1659,7 +1912,9 @@
           <cell r="B30" t="str">
             <v>Ochoa Duran Thalia</v>
           </cell>
-          <cell r="C30"/>
+          <cell r="C30">
+            <v>0</v>
+          </cell>
           <cell r="D30" t="str">
             <v>LU Florida</v>
           </cell>
@@ -1669,13 +1924,21 @@
           <cell r="F30" t="str">
             <v>42.00</v>
           </cell>
-          <cell r="G30"/>
-          <cell r="H30"/>
-          <cell r="I30"/>
+          <cell r="G30">
+            <v>0</v>
+          </cell>
+          <cell r="H30">
+            <v>0</v>
+          </cell>
+          <cell r="I30">
+            <v>0</v>
+          </cell>
           <cell r="J30" t="str">
             <v>NO</v>
           </cell>
-          <cell r="K30"/>
+          <cell r="K30">
+            <v>0</v>
+          </cell>
           <cell r="L30">
             <v>0</v>
           </cell>
@@ -1966,29 +2229,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:Q289"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="4"/>
-    <col min="2" max="2" width="9.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5546875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="10.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" style="4"/>
+    <col min="2" max="2" width="9.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.90625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.54296875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="10.453125" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" style="4" customWidth="1"/>
-    <col min="11" max="11" width="6.44140625" style="4" customWidth="1"/>
-    <col min="12" max="12" width="13.109375" style="4" customWidth="1"/>
-    <col min="13" max="13" width="7.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.44140625" style="4" customWidth="1"/>
-    <col min="15" max="15" width="6.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.5546875" style="4"/>
-    <col min="17" max="17" width="14.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="11.5546875" style="4"/>
+    <col min="9" max="9" width="11.453125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" style="4" customWidth="1"/>
+    <col min="11" max="11" width="6.453125" style="4" customWidth="1"/>
+    <col min="12" max="12" width="13.08984375" style="4" customWidth="1"/>
+    <col min="13" max="13" width="7.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.453125" style="4" customWidth="1"/>
+    <col min="15" max="15" width="6.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.54296875" style="4"/>
+    <col min="17" max="17" width="14.08984375" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="11.54296875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -2038,7 +2301,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>45901</v>
       </c>
@@ -2056,7 +2319,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>45901</v>
       </c>
@@ -2074,7 +2337,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>45901</v>
       </c>
@@ -2092,7 +2355,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>45901</v>
       </c>
@@ -2107,7 +2370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>45901</v>
       </c>
@@ -2122,7 +2385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>45901</v>
       </c>
@@ -2140,7 +2403,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>45901</v>
       </c>
@@ -2158,7 +2421,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>45901</v>
       </c>
@@ -2179,7 +2442,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>45901</v>
       </c>
@@ -2200,7 +2463,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>45901</v>
       </c>
@@ -2222,7 +2485,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>45901</v>
       </c>
@@ -2240,7 +2503,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>45901</v>
       </c>
@@ -2255,7 +2518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>45901</v>
       </c>
@@ -2276,7 +2539,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>45901</v>
       </c>
@@ -2297,7 +2560,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>45901</v>
       </c>
@@ -2315,7 +2578,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>45901</v>
       </c>
@@ -2333,7 +2596,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>45901</v>
       </c>
@@ -2348,7 +2611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>45901</v>
       </c>
@@ -2366,7 +2629,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>45901</v>
       </c>
@@ -2387,7 +2650,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>45901</v>
       </c>
@@ -2405,7 +2668,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>45901</v>
       </c>
@@ -2426,7 +2689,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>45901</v>
       </c>
@@ -2444,7 +2707,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>45901</v>
       </c>
@@ -2465,7 +2728,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>45901</v>
       </c>
@@ -2483,7 +2746,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>45931</v>
       </c>
@@ -2508,7 +2771,7 @@
         <v>9943.0976216535419</v>
       </c>
     </row>
-    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>45931</v>
       </c>
@@ -2533,7 +2796,7 @@
         <v>9845.2116900000001</v>
       </c>
     </row>
-    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>45931</v>
       </c>
@@ -2555,7 +2818,7 @@
         <v>9876.217631212121</v>
       </c>
     </row>
-    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>45931</v>
       </c>
@@ -2574,7 +2837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>45931</v>
       </c>
@@ -2596,7 +2859,7 @@
         <v>9792.8343385887092</v>
       </c>
     </row>
-    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>45931</v>
       </c>
@@ -2618,7 +2881,7 @@
         <v>10112.261986218487</v>
       </c>
     </row>
-    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>45931</v>
       </c>
@@ -2640,7 +2903,7 @@
         <v>9911.784182045456</v>
       </c>
     </row>
-    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>45931</v>
       </c>
@@ -2668,7 +2931,7 @@
         <v>9105.9318448800004</v>
       </c>
     </row>
-    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>45931</v>
       </c>
@@ -2690,7 +2953,7 @@
         <v>10263.705370338983</v>
       </c>
     </row>
-    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>45931</v>
       </c>
@@ -2712,7 +2975,7 @@
         <v>9611.4834238429758</v>
       </c>
     </row>
-    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>45931</v>
       </c>
@@ -2737,7 +3000,7 @@
         <v>9407.4009474408667</v>
       </c>
     </row>
-    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>45931</v>
       </c>
@@ -2762,7 +3025,7 @@
         <v>9155.460082272728</v>
       </c>
     </row>
-    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>45931</v>
       </c>
@@ -2784,7 +3047,7 @@
         <v>9659.5219028030297</v>
       </c>
     </row>
-    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>45931</v>
       </c>
@@ -2809,7 +3072,7 @@
         <v>9708.309949915254</v>
       </c>
     </row>
-    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>45931</v>
       </c>
@@ -2831,7 +3094,7 @@
         <v>9612.1727566086956</v>
       </c>
     </row>
-    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>45931</v>
       </c>
@@ -2856,7 +3119,7 @@
         <v>10483.191883990825</v>
       </c>
     </row>
-    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>45931</v>
       </c>
@@ -2881,7 +3144,7 @@
         <v>9567.2268119724758</v>
       </c>
     </row>
-    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>45931</v>
       </c>
@@ -2908,7 +3171,7 @@
         <v>9038.4294641666656</v>
       </c>
     </row>
-    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>45931</v>
       </c>
@@ -2930,7 +3193,7 @@
         <v>9126.4995916517855</v>
       </c>
     </row>
-    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>45931</v>
       </c>
@@ -2952,7 +3215,7 @@
         <v>9045.4182661538471</v>
       </c>
     </row>
-    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="3">
         <v>45931</v>
       </c>
@@ -2974,7 +3237,7 @@
         <v>8826.5215606836755</v>
       </c>
     </row>
-    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="3">
         <v>45931</v>
       </c>
@@ -2996,7 +3259,7 @@
         <v>8788.0516385393257</v>
       </c>
     </row>
-    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="3">
         <v>45931</v>
       </c>
@@ -3018,7 +3281,7 @@
         <v>8788.5621133333334</v>
       </c>
     </row>
-    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="3">
         <v>45931</v>
       </c>
@@ -3040,7 +3303,7 @@
         <v>8788.3031044886375</v>
       </c>
     </row>
-    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="3">
         <v>45931</v>
       </c>
@@ -3062,7 +3325,7 @@
         <v>8795.3369153731346</v>
       </c>
     </row>
-    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="3">
         <v>45931</v>
       </c>
@@ -3085,7 +3348,7 @@
         <v>8791.8473084210527</v>
       </c>
     </row>
-    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="3">
         <v>45931</v>
       </c>
@@ -3107,7 +3370,7 @@
         <v>8812.8832523809524</v>
       </c>
     </row>
-    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="3">
         <v>45962</v>
       </c>
@@ -3133,7 +3396,7 @@
       <c r="P53" s="6"/>
       <c r="Q53" s="7"/>
     </row>
-    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="3">
         <v>45962</v>
       </c>
@@ -3152,7 +3415,7 @@
       </c>
       <c r="P54" s="6"/>
     </row>
-    <row r="55" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="3">
         <v>45962</v>
       </c>
@@ -3171,7 +3434,7 @@
       </c>
       <c r="P55" s="6"/>
     </row>
-    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="3">
         <v>45962</v>
       </c>
@@ -3187,7 +3450,7 @@
       </c>
       <c r="P56" s="6"/>
     </row>
-    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="3">
         <v>45962</v>
       </c>
@@ -3206,7 +3469,7 @@
       </c>
       <c r="P57" s="6"/>
     </row>
-    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="3">
         <v>45962</v>
       </c>
@@ -3225,7 +3488,7 @@
       </c>
       <c r="P58" s="6"/>
     </row>
-    <row r="59" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="3">
         <v>45962</v>
       </c>
@@ -3244,7 +3507,7 @@
       </c>
       <c r="P59" s="6"/>
     </row>
-    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="3">
         <v>45962</v>
       </c>
@@ -3266,7 +3529,7 @@
       </c>
       <c r="P60" s="6"/>
     </row>
-    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="3">
         <v>45962</v>
       </c>
@@ -3285,7 +3548,7 @@
       </c>
       <c r="P61" s="6"/>
     </row>
-    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="3">
         <v>45962</v>
       </c>
@@ -3304,7 +3567,7 @@
       </c>
       <c r="P62" s="6"/>
     </row>
-    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="3">
         <v>45962</v>
       </c>
@@ -3326,7 +3589,7 @@
       </c>
       <c r="P63" s="6"/>
     </row>
-    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="3">
         <v>45962</v>
       </c>
@@ -3345,7 +3608,7 @@
       </c>
       <c r="P64" s="6"/>
     </row>
-    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="3">
         <v>45962</v>
       </c>
@@ -3367,7 +3630,7 @@
       </c>
       <c r="P65" s="6"/>
     </row>
-    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="3">
         <v>45962</v>
       </c>
@@ -3386,7 +3649,7 @@
       </c>
       <c r="P66" s="6"/>
     </row>
-    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="3">
         <v>45962</v>
       </c>
@@ -3405,7 +3668,7 @@
       </c>
       <c r="P67" s="6"/>
     </row>
-    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="3">
         <v>45962</v>
       </c>
@@ -3430,7 +3693,7 @@
       </c>
       <c r="P68" s="6"/>
     </row>
-    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="3">
         <v>45962</v>
       </c>
@@ -3452,7 +3715,7 @@
       </c>
       <c r="P69" s="6"/>
     </row>
-    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="3">
         <v>45962</v>
       </c>
@@ -3474,7 +3737,7 @@
       </c>
       <c r="P70" s="6"/>
     </row>
-    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="3">
         <v>45962</v>
       </c>
@@ -3493,7 +3756,7 @@
       </c>
       <c r="P71" s="6"/>
     </row>
-    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="3">
         <v>45962</v>
       </c>
@@ -3512,7 +3775,7 @@
       </c>
       <c r="P72" s="6"/>
     </row>
-    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="3">
         <v>45962</v>
       </c>
@@ -3534,7 +3797,7 @@
       </c>
       <c r="P73" s="6"/>
     </row>
-    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="3">
         <v>45962</v>
       </c>
@@ -3553,7 +3816,7 @@
       </c>
       <c r="P74" s="6"/>
     </row>
-    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="3">
         <v>45962</v>
       </c>
@@ -3572,7 +3835,7 @@
       </c>
       <c r="P75" s="6"/>
     </row>
-    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="3">
         <v>45962</v>
       </c>
@@ -3591,7 +3854,7 @@
       </c>
       <c r="P76" s="6"/>
     </row>
-    <row r="77" spans="1:16" s="5" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" s="5" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="3">
         <v>45962</v>
       </c>
@@ -3613,7 +3876,7 @@
       </c>
       <c r="P77" s="8"/>
     </row>
-    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="3">
         <v>45962</v>
       </c>
@@ -3632,7 +3895,7 @@
       </c>
       <c r="P78" s="6"/>
     </row>
-    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="3">
         <v>45962</v>
       </c>
@@ -3650,7 +3913,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="3">
         <v>45962</v>
       </c>
@@ -3671,7 +3934,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="81" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3">
         <v>45962</v>
       </c>
@@ -3692,7 +3955,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="82" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="3">
         <v>45962</v>
       </c>
@@ -3710,7 +3973,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="83" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="3">
         <v>45992</v>
       </c>
@@ -3732,7 +3995,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="84" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="3">
         <v>45992</v>
       </c>
@@ -3754,7 +4017,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="85" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="3">
         <v>45992</v>
       </c>
@@ -3772,7 +4035,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="86" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="3">
         <v>45992</v>
       </c>
@@ -3790,7 +4053,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="87" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="3">
         <v>45992</v>
       </c>
@@ -3808,7 +4071,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="88" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="3">
         <v>45992</v>
       </c>
@@ -3826,7 +4089,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="89" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="3">
         <v>45992</v>
       </c>
@@ -3844,7 +4107,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="90" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="3">
         <v>45992</v>
       </c>
@@ -3862,7 +4125,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="91" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="3">
         <v>45992</v>
       </c>
@@ -3880,7 +4143,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="92" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="3">
         <v>45992</v>
       </c>
@@ -3898,7 +4161,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="93" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="3">
         <v>45992</v>
       </c>
@@ -3919,7 +4182,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="94" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="3">
         <v>45992</v>
       </c>
@@ -3941,7 +4204,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="95" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="3">
         <v>45992</v>
       </c>
@@ -3963,7 +4226,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="96" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="3">
         <v>45992</v>
       </c>
@@ -3985,7 +4248,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="97" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="3">
         <v>45992</v>
       </c>
@@ -4006,7 +4269,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="98" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="3">
         <v>45992</v>
       </c>
@@ -4028,7 +4291,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="99" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="3">
         <v>45992</v>
       </c>
@@ -4053,7 +4316,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="100" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="3">
         <v>45992</v>
       </c>
@@ -4071,7 +4334,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="101" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="3">
         <v>45992</v>
       </c>
@@ -4089,7 +4352,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="102" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="3">
         <v>45992</v>
       </c>
@@ -4107,7 +4370,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="103" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="3">
         <v>45992</v>
       </c>
@@ -4125,7 +4388,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="104" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="3">
         <v>45992</v>
       </c>
@@ -4143,7 +4406,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="105" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="3">
         <v>45992</v>
       </c>
@@ -4161,7 +4424,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="106" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="3">
         <v>45992</v>
       </c>
@@ -4179,7 +4442,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="107" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="3">
         <v>45992</v>
       </c>
@@ -4197,7 +4460,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="108" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="3">
         <v>45992</v>
       </c>
@@ -4215,7 +4478,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="109" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="3">
         <v>45992</v>
       </c>
@@ -4233,7 +4496,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="110" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="3">
         <v>45992</v>
       </c>
@@ -4251,7 +4514,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="111" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="3">
         <v>45992</v>
       </c>
@@ -4269,7 +4532,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="112" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="3">
         <v>45992</v>
       </c>
@@ -4287,7 +4550,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="113" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="3">
         <v>45992</v>
       </c>
@@ -4305,7 +4568,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="114" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="3">
         <v>45992</v>
       </c>
@@ -4323,7 +4586,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="3">
         <v>46023</v>
       </c>
@@ -4344,7 +4607,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="3">
         <v>46023</v>
       </c>
@@ -4362,14 +4625,14 @@
         <v>102</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="3">
         <v>46023</v>
       </c>
       <c r="B117" s="4">
         <v>10</v>
       </c>
-      <c r="C117" s="4" t="s">
+      <c r="C117" s="5" t="s">
         <v>8</v>
       </c>
       <c r="L117" s="4">
@@ -4383,7 +4646,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="3">
         <v>46023</v>
       </c>
@@ -4401,14 +4664,14 @@
         <v>100</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="3">
         <v>46023</v>
       </c>
       <c r="B119" s="4">
         <v>32</v>
       </c>
-      <c r="C119" s="4" t="s">
+      <c r="C119" s="5" t="s">
         <v>29</v>
       </c>
       <c r="L119" s="4">
@@ -4422,7 +4685,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="3">
         <v>46023</v>
       </c>
@@ -4440,7 +4703,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="3">
         <v>46023</v>
       </c>
@@ -4458,7 +4721,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="3">
         <v>46023</v>
       </c>
@@ -4476,14 +4739,14 @@
         <v>119</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="3">
         <v>46023</v>
       </c>
       <c r="B123" s="4">
         <v>36</v>
       </c>
-      <c r="C123" s="4" t="s">
+      <c r="C123" s="5" t="s">
         <v>32</v>
       </c>
       <c r="M123" s="4">
@@ -4497,7 +4760,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="3">
         <v>46023</v>
       </c>
@@ -4515,7 +4778,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="3">
         <v>46023</v>
       </c>
@@ -4533,7 +4796,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="3">
         <v>46023</v>
       </c>
@@ -4551,7 +4814,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="3">
         <v>46023</v>
       </c>
@@ -4569,7 +4832,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="3">
         <v>46023</v>
       </c>
@@ -4591,7 +4854,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="3">
         <v>46023</v>
       </c>
@@ -4609,7 +4872,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="3">
         <v>46023</v>
       </c>
@@ -4622,15 +4885,12 @@
       <c r="K130" s="4">
         <v>87</v>
       </c>
-      <c r="N130" s="4">
-        <v>28</v>
-      </c>
       <c r="O130" s="12">
         <f t="shared" si="1"/>
-        <v>115</v>
-      </c>
-    </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="131" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="3">
         <v>46023</v>
       </c>
@@ -4647,14 +4907,14 @@
         <v>116</v>
       </c>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="3">
         <v>46023</v>
       </c>
       <c r="B132" s="4">
         <v>29</v>
       </c>
-      <c r="C132" s="4" t="s">
+      <c r="C132" s="5" t="s">
         <v>20</v>
       </c>
       <c r="K132" s="4">
@@ -4664,18 +4924,18 @@
         <v>56</v>
       </c>
       <c r="O132" s="12">
-        <f t="shared" ref="O131:O195" si="2">SUM(D132:N132)</f>
+        <f t="shared" ref="O132:O195" si="2">SUM(D132:N132)</f>
         <v>116</v>
       </c>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="3">
         <v>46023</v>
       </c>
       <c r="B133" s="4">
         <v>1</v>
       </c>
-      <c r="C133" s="4" t="s">
+      <c r="C133" s="5" t="s">
         <v>3</v>
       </c>
       <c r="E133" s="4">
@@ -4692,7 +4952,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="3">
         <v>46023</v>
       </c>
@@ -4708,15 +4968,13 @@
       <c r="H134" s="4">
         <v>12</v>
       </c>
-      <c r="N134" s="5">
-        <v>12</v>
-      </c>
+      <c r="N134" s="5"/>
       <c r="O134" s="12">
         <f t="shared" si="2"/>
-        <v>116</v>
-      </c>
-    </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="135" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="3">
         <v>46023</v>
       </c>
@@ -4737,14 +4995,14 @@
         <v>111</v>
       </c>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="3">
         <v>46023</v>
       </c>
       <c r="B136" s="4">
         <v>40</v>
       </c>
-      <c r="C136" s="4" t="s">
+      <c r="C136" s="5" t="s">
         <v>36</v>
       </c>
       <c r="F136" s="4">
@@ -4761,7 +5019,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="3">
         <v>46023</v>
       </c>
@@ -4779,14 +5037,14 @@
         <v>102</v>
       </c>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="3">
         <v>46023</v>
       </c>
       <c r="B138" s="4">
         <v>3</v>
       </c>
-      <c r="C138" s="4" t="s">
+      <c r="C138" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E138" s="4">
@@ -4796,14 +5054,14 @@
         <v>18</v>
       </c>
       <c r="N138" s="5">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="O138" s="12">
         <f t="shared" si="2"/>
-        <v>121</v>
-      </c>
-    </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="139" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="3">
         <v>46023</v>
       </c>
@@ -4821,7 +5079,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="3">
         <v>46023</v>
       </c>
@@ -4839,7 +5097,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="3">
         <v>46023</v>
       </c>
@@ -4849,15 +5107,12 @@
       <c r="C141" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="N141" s="4">
-        <v>44</v>
-      </c>
       <c r="O141" s="12">
         <f t="shared" si="2"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" s="3">
         <v>46023</v>
       </c>
@@ -4875,7 +5130,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="3">
         <v>46023</v>
       </c>
@@ -4893,7 +5148,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="3">
         <v>46023</v>
       </c>
@@ -4911,7 +5166,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="3">
         <v>46023</v>
       </c>
@@ -4929,14 +5184,14 @@
         <v>122</v>
       </c>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="3">
         <v>46023</v>
       </c>
       <c r="B146" s="4">
         <v>39</v>
       </c>
-      <c r="C146" s="4" t="s">
+      <c r="C146" s="5" t="s">
         <v>35</v>
       </c>
       <c r="J146" s="4">
@@ -4950,7 +5205,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="3">
         <v>46023</v>
       </c>
@@ -4971,7 +5226,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="148" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="3">
         <v>46054</v>
       </c>
@@ -4995,7 +5250,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="149" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="3">
         <v>46054</v>
       </c>
@@ -5013,7 +5268,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="150" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="3">
         <v>46054</v>
       </c>
@@ -5031,7 +5286,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="151" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" s="3">
         <v>46054</v>
       </c>
@@ -5044,12 +5299,15 @@
       <c r="L151" s="4">
         <v>44</v>
       </c>
+      <c r="N151" s="4">
+        <v>56</v>
+      </c>
       <c r="O151" s="4">
         <f t="shared" si="2"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="152" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="152" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" s="3">
         <v>46054</v>
       </c>
@@ -5067,7 +5325,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="153" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" s="3">
         <v>46054</v>
       </c>
@@ -5085,7 +5343,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="154" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" s="3">
         <v>46054</v>
       </c>
@@ -5098,12 +5356,15 @@
       <c r="M154" s="4">
         <v>70</v>
       </c>
+      <c r="N154" s="4">
+        <v>56</v>
+      </c>
       <c r="O154" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="155" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="155" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" s="3">
         <v>46054</v>
       </c>
@@ -5121,7 +5382,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="156" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" s="3">
         <v>46054</v>
       </c>
@@ -5134,12 +5395,15 @@
       <c r="M156" s="4">
         <v>84</v>
       </c>
+      <c r="N156" s="4">
+        <v>12</v>
+      </c>
       <c r="O156" s="4">
         <f t="shared" si="2"/>
-        <v>84</v>
-      </c>
-    </row>
-    <row r="157" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="157" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" s="3">
         <v>46054</v>
       </c>
@@ -5152,12 +5416,18 @@
       <c r="D157" s="4">
         <v>80</v>
       </c>
+      <c r="N157" s="4">
+        <v>56</v>
+      </c>
       <c r="O157" s="4">
         <f t="shared" si="2"/>
-        <v>80</v>
-      </c>
-    </row>
-    <row r="158" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+      <c r="Q157" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="158" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="3">
         <v>46054</v>
       </c>
@@ -5175,7 +5445,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="159" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="3">
         <v>46054</v>
       </c>
@@ -5193,7 +5463,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="160" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" s="3">
         <v>46054</v>
       </c>
@@ -5215,7 +5485,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="161" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" s="3">
         <v>46054</v>
       </c>
@@ -5233,7 +5503,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="162" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" s="3">
         <v>46054</v>
       </c>
@@ -5254,7 +5524,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="163" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" s="3">
         <v>46054</v>
       </c>
@@ -5272,7 +5542,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="164" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" s="3">
         <v>46054</v>
       </c>
@@ -5290,7 +5560,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="165" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" s="3">
         <v>46054</v>
       </c>
@@ -5308,7 +5578,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="166" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" s="3">
         <v>46054</v>
       </c>
@@ -5329,7 +5599,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="167" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" s="3">
         <v>46054</v>
       </c>
@@ -5345,12 +5615,18 @@
       <c r="M167" s="4">
         <v>14</v>
       </c>
+      <c r="N167" s="4">
+        <v>56</v>
+      </c>
       <c r="O167" s="4">
         <f t="shared" si="2"/>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="168" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+      <c r="Q167" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="168" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" s="3">
         <v>46054</v>
       </c>
@@ -5371,7 +5647,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="169" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" s="3">
         <v>46054</v>
       </c>
@@ -5392,7 +5668,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="170" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" s="3">
         <v>46054</v>
       </c>
@@ -5410,7 +5686,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="171" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" s="3">
         <v>46054</v>
       </c>
@@ -5428,7 +5704,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="172" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" s="3">
         <v>46054</v>
       </c>
@@ -5441,12 +5717,15 @@
       <c r="H172" s="4">
         <v>43</v>
       </c>
+      <c r="N172" s="4">
+        <v>56</v>
+      </c>
       <c r="O172" s="4">
         <f t="shared" si="2"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="173" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="173" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" s="3">
         <v>46054</v>
       </c>
@@ -5464,7 +5743,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="174" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" s="3">
         <v>46054</v>
       </c>
@@ -5485,7 +5764,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="175" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" s="3">
         <v>46054</v>
       </c>
@@ -5503,7 +5782,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="176" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" s="3">
         <v>46054</v>
       </c>
@@ -5524,7 +5803,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="177" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="3">
         <v>46054</v>
       </c>
@@ -5542,7 +5821,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="178" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" s="3">
         <v>46054</v>
       </c>
@@ -5566,7 +5845,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="179" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" s="3">
         <v>46082</v>
       </c>
@@ -5579,12 +5858,15 @@
       <c r="L179" s="4">
         <v>89</v>
       </c>
+      <c r="N179" s="4">
+        <v>36</v>
+      </c>
       <c r="O179" s="4">
         <f t="shared" si="2"/>
-        <v>89</v>
-      </c>
-    </row>
-    <row r="180" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="180" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" s="3">
         <v>46082</v>
       </c>
@@ -5602,7 +5884,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="181" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="3">
         <v>46082</v>
       </c>
@@ -5620,7 +5902,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="182" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" s="3">
         <v>46082</v>
       </c>
@@ -5638,7 +5920,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="183" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="3">
         <v>46082</v>
       </c>
@@ -5656,7 +5938,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="184" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" s="3">
         <v>46082</v>
       </c>
@@ -5677,7 +5959,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="185" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" s="3">
         <v>46082</v>
       </c>
@@ -5695,7 +5977,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="186" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" s="3">
         <v>46082</v>
       </c>
@@ -5708,12 +5990,15 @@
       <c r="D186" s="4">
         <v>109</v>
       </c>
+      <c r="N186" s="4">
+        <v>12</v>
+      </c>
       <c r="O186" s="4">
         <f t="shared" si="2"/>
-        <v>109</v>
-      </c>
-    </row>
-    <row r="187" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="187" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" s="3">
         <v>46082</v>
       </c>
@@ -5731,7 +6016,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="188" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" s="3">
         <v>46082</v>
       </c>
@@ -5752,7 +6037,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="189" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" s="3">
         <v>46082</v>
       </c>
@@ -5773,7 +6058,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="190" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" s="3">
         <v>46082</v>
       </c>
@@ -5791,7 +6076,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="191" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" s="3">
         <v>46082</v>
       </c>
@@ -5809,7 +6094,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="192" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" s="3">
         <v>46082</v>
       </c>
@@ -5827,7 +6112,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="193" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" s="3">
         <v>46082</v>
       </c>
@@ -5848,7 +6133,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="194" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" s="3">
         <v>46082</v>
       </c>
@@ -5863,7 +6148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" s="3">
         <v>46082</v>
       </c>
@@ -5884,7 +6169,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="196" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" s="3">
         <v>46082</v>
       </c>
@@ -5908,7 +6193,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="197" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" s="3">
         <v>46082</v>
       </c>
@@ -5929,7 +6214,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="198" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" s="3">
         <v>46082</v>
       </c>
@@ -5944,7 +6229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" s="3">
         <v>46082</v>
       </c>
@@ -5962,7 +6247,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="200" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" s="3">
         <v>46082</v>
       </c>
@@ -5975,12 +6260,15 @@
       <c r="H200" s="4">
         <v>66</v>
       </c>
+      <c r="N200" s="4">
+        <v>56</v>
+      </c>
       <c r="O200" s="4">
         <f t="shared" si="3"/>
-        <v>66</v>
-      </c>
-    </row>
-    <row r="201" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="201" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" s="3">
         <v>46082</v>
       </c>
@@ -5998,7 +6286,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="202" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" s="3">
         <v>46082</v>
       </c>
@@ -6011,12 +6299,15 @@
       <c r="I202" s="4">
         <v>69</v>
       </c>
+      <c r="N202" s="4">
+        <v>56</v>
+      </c>
       <c r="O202" s="4">
         <f t="shared" si="3"/>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="203" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="203" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" s="3">
         <v>46082</v>
       </c>
@@ -6034,7 +6325,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="204" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" s="3">
         <v>46082</v>
       </c>
@@ -6055,7 +6346,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="205" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" s="3">
         <v>46082</v>
       </c>
@@ -6073,7 +6364,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="206" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" s="3">
         <v>46082</v>
       </c>
@@ -6094,7 +6385,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="207" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" s="3">
         <v>46113</v>
       </c>
@@ -6115,7 +6406,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="208" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" s="3">
         <v>46113</v>
       </c>
@@ -6133,7 +6424,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="209" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" s="3">
         <v>46113</v>
       </c>
@@ -6151,7 +6442,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="210" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" s="3">
         <v>46113</v>
       </c>
@@ -6169,7 +6460,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="211" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" s="3">
         <v>46113</v>
       </c>
@@ -6187,7 +6478,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="212" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" s="3">
         <v>46113</v>
       </c>
@@ -6208,7 +6499,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="213" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" s="3">
         <v>46113</v>
       </c>
@@ -6226,7 +6517,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="214" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" s="3">
         <v>46113</v>
       </c>
@@ -6244,7 +6535,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="215" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" s="3">
         <v>46113</v>
       </c>
@@ -6265,7 +6556,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="216" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" s="3">
         <v>46113</v>
       </c>
@@ -6283,7 +6574,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="217" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" s="3">
         <v>46113</v>
       </c>
@@ -6301,7 +6592,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="218" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" s="3">
         <v>46113</v>
       </c>
@@ -6319,7 +6610,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="219" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" s="3">
         <v>46113</v>
       </c>
@@ -6340,7 +6631,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="220" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" s="3">
         <v>46113</v>
       </c>
@@ -6361,7 +6652,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="221" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" s="3">
         <v>46113</v>
       </c>
@@ -6379,7 +6670,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="222" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" s="3">
         <v>46113</v>
       </c>
@@ -6397,7 +6688,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="223" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" s="3">
         <v>46113</v>
       </c>
@@ -6415,7 +6706,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="224" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" s="3">
         <v>46113</v>
       </c>
@@ -6433,7 +6724,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="225" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" s="3">
         <v>46113</v>
       </c>
@@ -6451,7 +6742,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="226" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" s="3">
         <v>46113</v>
       </c>
@@ -6472,7 +6763,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="227" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" s="3">
         <v>46113</v>
       </c>
@@ -6490,7 +6781,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="228" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" s="3">
         <v>46113</v>
       </c>
@@ -6511,7 +6802,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="229" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" s="3">
         <v>46113</v>
       </c>
@@ -6529,7 +6820,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="230" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" s="3">
         <v>46113</v>
       </c>
@@ -6547,7 +6838,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="231" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" s="3">
         <v>46113</v>
       </c>
@@ -6565,7 +6856,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="232" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" s="3">
         <v>46113</v>
       </c>
@@ -6586,7 +6877,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="233" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" s="3">
         <v>46113</v>
       </c>
@@ -6604,7 +6895,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="234" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" s="3">
         <v>46113</v>
       </c>
@@ -6622,7 +6913,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="235" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" s="3">
         <v>46143</v>
       </c>
@@ -6643,7 +6934,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="236" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" s="3">
         <v>46143</v>
       </c>
@@ -6661,7 +6952,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="237" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" s="3">
         <v>46143</v>
       </c>
@@ -6679,7 +6970,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="238" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" s="3">
         <v>46143</v>
       </c>
@@ -6697,7 +6988,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="239" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" s="3">
         <v>46143</v>
       </c>
@@ -6715,7 +7006,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="240" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" s="3">
         <v>46143</v>
       </c>
@@ -6733,7 +7024,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="241" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" s="3">
         <v>46143</v>
       </c>
@@ -6751,7 +7042,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="242" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" s="3">
         <v>46143</v>
       </c>
@@ -6775,7 +7066,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="243" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" s="3">
         <v>46143</v>
       </c>
@@ -6793,7 +7084,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="244" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" s="3">
         <v>46143</v>
       </c>
@@ -6811,7 +7102,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="245" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" s="3">
         <v>46143</v>
       </c>
@@ -6829,7 +7120,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="246" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" s="3">
         <v>46143</v>
       </c>
@@ -6847,7 +7138,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="247" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" s="3">
         <v>46143</v>
       </c>
@@ -6868,7 +7159,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="248" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" s="3">
         <v>46143</v>
       </c>
@@ -6886,7 +7177,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="249" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" s="3">
         <v>46143</v>
       </c>
@@ -6907,7 +7198,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="250" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" s="3">
         <v>46143</v>
       </c>
@@ -6928,7 +7219,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="251" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" s="3">
         <v>46143</v>
       </c>
@@ -6949,7 +7240,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="252" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" s="3">
         <v>46143</v>
       </c>
@@ -6967,7 +7258,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="253" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" s="3">
         <v>46143</v>
       </c>
@@ -6985,7 +7276,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="254" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" s="3">
         <v>46143</v>
       </c>
@@ -7006,7 +7297,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="255" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" s="3">
         <v>46143</v>
       </c>
@@ -7024,7 +7315,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="256" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" s="3">
         <v>46143</v>
       </c>
@@ -7042,7 +7333,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="257" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A257" s="3">
         <v>46143</v>
       </c>
@@ -7066,7 +7357,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="258" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" s="3">
         <v>46143</v>
       </c>
@@ -7084,7 +7375,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="259" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" s="3">
         <v>46143</v>
       </c>
@@ -7105,7 +7396,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="260" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A260" s="3">
         <v>46143</v>
       </c>
@@ -7126,7 +7417,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="261" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" s="3">
         <v>46143</v>
       </c>
@@ -7144,7 +7435,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="262" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A262" s="3">
         <v>46174</v>
       </c>
@@ -7162,7 +7453,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="263" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A263" s="3">
         <v>46174</v>
       </c>
@@ -7180,7 +7471,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="264" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A264" s="3">
         <v>46174</v>
       </c>
@@ -7198,7 +7489,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="265" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A265" s="3">
         <v>46174</v>
       </c>
@@ -7216,7 +7507,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="266" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A266" s="3">
         <v>46174</v>
       </c>
@@ -7227,14 +7518,14 @@
         <v>10</v>
       </c>
       <c r="H266" s="4">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="O266" s="4">
         <f t="shared" si="4"/>
-        <v>121</v>
-      </c>
-    </row>
-    <row r="267" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="267" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A267" s="3">
         <v>46174</v>
       </c>
@@ -7255,7 +7546,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="268" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A268" s="3">
         <v>46174</v>
       </c>
@@ -7273,7 +7564,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="269" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A269" s="3">
         <v>46174</v>
       </c>
@@ -7294,7 +7585,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="270" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A270" s="3">
         <v>46174</v>
       </c>
@@ -7312,7 +7603,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="271" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A271" s="3">
         <v>46174</v>
       </c>
@@ -7330,7 +7621,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="272" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A272" s="3">
         <v>46174</v>
       </c>
@@ -7348,7 +7639,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="273" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A273" s="3">
         <v>46174</v>
       </c>
@@ -7366,7 +7657,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="274" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A274" s="3">
         <v>46174</v>
       </c>
@@ -7387,7 +7678,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="275" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A275" s="3">
         <v>46174</v>
       </c>
@@ -7405,7 +7696,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="276" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A276" s="3">
         <v>46174</v>
       </c>
@@ -7426,7 +7717,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="277" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A277" s="3">
         <v>46174</v>
       </c>
@@ -7447,7 +7738,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="278" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A278" s="3">
         <v>46174</v>
       </c>
@@ -7465,7 +7756,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="279" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A279" s="3">
         <v>46174</v>
       </c>
@@ -7478,15 +7769,12 @@
       <c r="D279" s="4">
         <v>118</v>
       </c>
-      <c r="N279" s="4">
-        <v>8</v>
-      </c>
       <c r="O279" s="4">
         <f t="shared" si="4"/>
-        <v>126</v>
-      </c>
-    </row>
-    <row r="280" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="280" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A280" s="3">
         <v>46174</v>
       </c>
@@ -7504,7 +7792,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="281" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A281" s="3">
         <v>46174</v>
       </c>
@@ -7522,7 +7810,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="282" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A282" s="3">
         <v>46174</v>
       </c>
@@ -7533,14 +7821,17 @@
         <v>59</v>
       </c>
       <c r="F282" s="4">
-        <v>120</v>
+        <v>112</v>
+      </c>
+      <c r="M282" s="4">
+        <v>8</v>
       </c>
       <c r="O282" s="4">
         <f t="shared" si="4"/>
         <v>120</v>
       </c>
     </row>
-    <row r="283" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A283" s="3">
         <v>46174</v>
       </c>
@@ -7558,7 +7849,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="284" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A284" s="3">
         <v>46174</v>
       </c>
@@ -7579,7 +7870,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="285" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A285" s="3">
         <v>46174</v>
       </c>
@@ -7589,18 +7880,18 @@
       <c r="C285" s="4" t="s">
         <v>65</v>
       </c>
+      <c r="E285" s="4">
+        <v>81</v>
+      </c>
       <c r="F285" s="4">
         <v>30</v>
-      </c>
-      <c r="M285" s="4">
-        <v>81</v>
       </c>
       <c r="O285" s="4">
         <f t="shared" si="4"/>
         <v>111</v>
       </c>
     </row>
-    <row r="286" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A286" s="3">
         <v>46174</v>
       </c>
@@ -7618,7 +7909,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="287" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A287" s="3">
         <v>46174</v>
       </c>
@@ -7639,7 +7930,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="288" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A288" s="3">
         <v>46174</v>
       </c>
@@ -7657,17 +7948,14 @@
         <v>14</v>
       </c>
     </row>
-    <row r="289" spans="15:15" x14ac:dyDescent="0.3">
-      <c r="O289" s="5">
-        <f>SUBTOTAL(9,O2:O288)</f>
-        <v>3538</v>
-      </c>
+    <row r="289" spans="15:15" x14ac:dyDescent="0.35">
+      <c r="O289" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:P288">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="1" dateTimeGrouping="month"/>
+        <dateGroupItem year="2026" month="6" dateTimeGrouping="month"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -7678,12 +7966,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -7703,7 +7991,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -7717,7 +8005,7 @@
         <v>46088</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>3</v>
       </c>
@@ -7728,7 +8016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>4</v>
       </c>
@@ -7739,7 +8027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>10</v>
       </c>
@@ -7750,7 +8038,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>11</v>
       </c>
@@ -7761,7 +8049,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>12</v>
       </c>
@@ -7772,7 +8060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>13</v>
       </c>
@@ -7783,7 +8071,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>14</v>
       </c>
@@ -7794,7 +8082,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>15</v>
       </c>
@@ -7805,7 +8093,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>18</v>
       </c>
@@ -7816,7 +8104,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>19</v>
       </c>
@@ -7827,7 +8115,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>20</v>
       </c>
@@ -7838,7 +8126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <v>21</v>
       </c>
@@ -7852,7 +8140,7 @@
         <v>46034</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <v>27</v>
       </c>
@@ -7863,7 +8151,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <v>28</v>
       </c>
@@ -7874,7 +8162,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>29</v>
       </c>
@@ -7892,7 +8180,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>30</v>
       </c>
@@ -7906,7 +8194,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>31</v>
       </c>
@@ -7917,7 +8205,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>32</v>
       </c>
@@ -7931,7 +8219,7 @@
         <v>46076</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>34</v>
       </c>
@@ -7945,7 +8233,7 @@
         <v>45998</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
         <v>36</v>
       </c>
@@ -7956,7 +8244,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
         <v>38</v>
       </c>
@@ -7970,7 +8258,7 @@
         <v>46123</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
         <v>39</v>
       </c>
@@ -7988,7 +8276,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
         <v>40</v>
       </c>
@@ -8002,7 +8290,7 @@
         <v>46123</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
         <v>41</v>
       </c>
@@ -8019,7 +8307,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="4">
         <v>42</v>
       </c>
@@ -8030,7 +8318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>43</v>
       </c>
@@ -8044,7 +8332,7 @@
         <v>46007</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="4">
         <v>44</v>
       </c>
@@ -8064,7 +8352,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="4">
         <v>45</v>
       </c>
@@ -8078,7 +8366,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="4">
         <v>46</v>
       </c>
@@ -8092,7 +8380,7 @@
         <v>46097</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="4">
         <v>47</v>
       </c>
@@ -8106,7 +8394,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="4">
         <v>49</v>
       </c>
@@ -8117,7 +8405,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>51</v>
       </c>
@@ -8131,7 +8419,7 @@
         <v>46032</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="4">
         <v>52</v>
       </c>
@@ -8142,7 +8430,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="4">
         <v>53</v>
       </c>
@@ -8156,7 +8444,7 @@
         <v>46076</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="4">
         <v>54</v>
       </c>
@@ -8167,7 +8455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="4">
         <v>55</v>
       </c>
@@ -8181,7 +8469,7 @@
         <v>46119</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="4">
         <v>58</v>
       </c>
@@ -8193,7 +8481,7 @@
       </c>
       <c r="D39" s="10"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="4">
         <v>63</v>
       </c>

</xml_diff>

<commit_message>
creación de tablero de resultados para Carlos. Actualización archivos para nuevo presupuesto y reporte de gastos mensual julio 2026
</commit_message>
<xml_diff>
--- a/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
+++ b/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="75">
   <si>
     <t>Florida</t>
   </si>
@@ -251,6 +251,9 @@
   </si>
   <si>
     <t>las horas son del recibo, no estaban en el excel. Se desvinculó este mes</t>
+  </si>
+  <si>
+    <t>No le sumo 2 días injustificados que se le descontaron</t>
   </si>
 </sst>
 </file>
@@ -626,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P289"/>
+  <dimension ref="A1:P314"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="4"/>
@@ -5694,7 +5697,7 @@
         <v>65</v>
       </c>
       <c r="O260" s="4">
-        <f t="shared" ref="O260:O288" si="4">SUM(D260:N260)</f>
+        <f t="shared" ref="O260:O314" si="4">SUM(D260:N260)</f>
         <v>82</v>
       </c>
     </row>
@@ -6229,8 +6232,506 @@
         <v>14</v>
       </c>
     </row>
-    <row r="289" spans="15:15" x14ac:dyDescent="0.3">
-      <c r="O289" s="5"/>
+    <row r="289" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A289" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B289" s="4">
+        <v>3</v>
+      </c>
+      <c r="C289" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D289" s="4">
+        <v>117</v>
+      </c>
+      <c r="O289" s="4">
+        <f t="shared" si="4"/>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="290" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A290" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B290" s="4">
+        <v>4</v>
+      </c>
+      <c r="C290" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D290" s="4">
+        <v>132</v>
+      </c>
+      <c r="O290" s="4">
+        <f t="shared" si="4"/>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="291" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A291" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B291" s="4">
+        <v>10</v>
+      </c>
+      <c r="C291" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L291" s="4">
+        <v>108</v>
+      </c>
+      <c r="O291" s="4">
+        <f t="shared" si="4"/>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="292" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A292" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B292" s="4">
+        <v>11</v>
+      </c>
+      <c r="C292" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I292" s="4">
+        <v>118</v>
+      </c>
+      <c r="O292" s="4">
+        <f t="shared" si="4"/>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="293" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A293" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B293" s="4">
+        <v>12</v>
+      </c>
+      <c r="C293" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H293" s="4">
+        <v>118</v>
+      </c>
+      <c r="O293" s="4">
+        <f t="shared" si="4"/>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="294" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A294" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B294" s="4">
+        <v>14</v>
+      </c>
+      <c r="C294" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I294" s="4">
+        <v>80</v>
+      </c>
+      <c r="K294" s="4">
+        <v>16</v>
+      </c>
+      <c r="N294" s="4">
+        <v>16</v>
+      </c>
+      <c r="O294" s="4">
+        <f t="shared" si="4"/>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="295" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A295" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B295" s="4">
+        <v>15</v>
+      </c>
+      <c r="C295" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L295" s="4">
+        <v>100</v>
+      </c>
+      <c r="O295" s="4">
+        <f t="shared" si="4"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="296" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A296" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B296" s="4">
+        <v>18</v>
+      </c>
+      <c r="C296" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D296" s="4">
+        <v>22</v>
+      </c>
+      <c r="E296" s="5">
+        <v>83</v>
+      </c>
+      <c r="O296" s="4">
+        <f t="shared" si="4"/>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="297" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A297" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B297" s="4">
+        <v>19</v>
+      </c>
+      <c r="C297" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F297" s="4">
+        <v>42</v>
+      </c>
+      <c r="M297" s="4">
+        <v>86</v>
+      </c>
+      <c r="O297" s="4">
+        <f t="shared" si="4"/>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="298" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A298" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B298" s="4">
+        <v>20</v>
+      </c>
+      <c r="C298" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H298" s="4">
+        <v>116</v>
+      </c>
+      <c r="O298" s="4">
+        <f t="shared" si="4"/>
+        <v>116</v>
+      </c>
+    </row>
+    <row r="299" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A299" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B299" s="4">
+        <v>27</v>
+      </c>
+      <c r="C299" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K299" s="4">
+        <v>95</v>
+      </c>
+      <c r="O299" s="4">
+        <f t="shared" si="4"/>
+        <v>95</v>
+      </c>
+      <c r="P299" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="300" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A300" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B300" s="4">
+        <v>28</v>
+      </c>
+      <c r="C300" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K300" s="4">
+        <v>114</v>
+      </c>
+      <c r="O300" s="4">
+        <f t="shared" si="4"/>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="301" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A301" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B301" s="4">
+        <v>29</v>
+      </c>
+      <c r="C301" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J301" s="4">
+        <v>96</v>
+      </c>
+      <c r="K301" s="4">
+        <v>14</v>
+      </c>
+      <c r="O301" s="4">
+        <f t="shared" si="4"/>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="302" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A302" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B302" s="4">
+        <v>31</v>
+      </c>
+      <c r="C302" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J302" s="4">
+        <v>108</v>
+      </c>
+      <c r="O302" s="4">
+        <f t="shared" si="4"/>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="303" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A303" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B303" s="4">
+        <v>36</v>
+      </c>
+      <c r="C303" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F303" s="4">
+        <v>49</v>
+      </c>
+      <c r="M303" s="4">
+        <v>76</v>
+      </c>
+      <c r="O303" s="4">
+        <f t="shared" si="4"/>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="304" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A304" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B304" s="4">
+        <v>39</v>
+      </c>
+      <c r="C304" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I304" s="4">
+        <v>101</v>
+      </c>
+      <c r="K304" s="5">
+        <v>14</v>
+      </c>
+      <c r="O304" s="4">
+        <f t="shared" si="4"/>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="305" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A305" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B305" s="4">
+        <v>41</v>
+      </c>
+      <c r="C305" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M305" s="4">
+        <v>125</v>
+      </c>
+      <c r="O305" s="4">
+        <f t="shared" si="4"/>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="306" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A306" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B306" s="4">
+        <v>42</v>
+      </c>
+      <c r="C306" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D306" s="4">
+        <v>127</v>
+      </c>
+      <c r="O306" s="4">
+        <f t="shared" si="4"/>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="307" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A307" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B307" s="4">
+        <v>49</v>
+      </c>
+      <c r="C307" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="J307" s="4">
+        <v>104</v>
+      </c>
+      <c r="O307" s="4">
+        <f t="shared" si="4"/>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="308" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A308" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B308" s="4">
+        <v>52</v>
+      </c>
+      <c r="C308" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="L308" s="4">
+        <v>88</v>
+      </c>
+      <c r="O308" s="4">
+        <f t="shared" si="4"/>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="309" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A309" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B309" s="4">
+        <v>54</v>
+      </c>
+      <c r="C309" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F309" s="4">
+        <v>103</v>
+      </c>
+      <c r="M309" s="4">
+        <v>17</v>
+      </c>
+      <c r="O309" s="4">
+        <f t="shared" si="4"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="310" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A310" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B310" s="4">
+        <v>58</v>
+      </c>
+      <c r="C310" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D310" s="4">
+        <v>118</v>
+      </c>
+      <c r="O310" s="4">
+        <f t="shared" si="4"/>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="311" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A311" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B311" s="4">
+        <v>59</v>
+      </c>
+      <c r="C311" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="M311" s="4">
+        <v>17</v>
+      </c>
+      <c r="O311" s="4">
+        <f t="shared" si="4"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="312" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A312" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B312" s="4">
+        <v>60</v>
+      </c>
+      <c r="C312" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D312" s="4">
+        <v>22</v>
+      </c>
+      <c r="E312" s="5">
+        <v>84</v>
+      </c>
+      <c r="O312" s="4">
+        <f t="shared" si="4"/>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="313" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A313" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B313" s="4">
+        <v>61</v>
+      </c>
+      <c r="C313" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H313" s="4">
+        <v>119</v>
+      </c>
+      <c r="O313" s="4">
+        <f t="shared" si="4"/>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="314" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A314" s="3">
+        <v>46204</v>
+      </c>
+      <c r="B314" s="4">
+        <v>62</v>
+      </c>
+      <c r="C314" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F314" s="4">
+        <v>61</v>
+      </c>
+      <c r="M314" s="4">
+        <v>64</v>
+      </c>
+      <c r="O314" s="4">
+        <f t="shared" si="4"/>
+        <v>125</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O288"/>
@@ -6240,7 +6741,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="21.33203125" bestFit="1" customWidth="1"/>
@@ -6761,21 +7262,35 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
+        <v>59</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="C40" t="s">
+        <v>55</v>
+      </c>
+      <c r="D40" s="8">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="4">
+        <v>63</v>
+      </c>
+      <c r="B41" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C41" t="s">
         <v>0</v>
       </c>
-      <c r="D40" s="8">
+      <c r="D41" s="8">
         <v>46185</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F40"/>
-  <sortState ref="A2:B169">
+  <sortState ref="A2:F41">
     <sortCondition ref="A1"/>
   </sortState>
   <conditionalFormatting sqref="A1:A1048576">

</xml_diff>

<commit_message>
seguí completando los gastos
</commit_message>
<xml_diff>
--- a/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
+++ b/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maval\Documents\Vale laburo\Castelli\Reportes\Reporte_gastos\Sueldos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Valeria\Reportes\Reporte_gastos\Sueldos\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6312"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6310"/>
   </bookViews>
   <sheets>
     <sheet name="tabla x hora" sheetId="1" r:id="rId1"/>
     <sheet name="vendedora-tienda" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tabla x hora'!$A$1:$O$288</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tabla x hora'!$A$1:$O$315</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'vendedora-tienda'!$A$1:$F$40</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="76">
   <si>
     <t>Florida</t>
   </si>
@@ -254,6 +254,9 @@
   </si>
   <si>
     <t>No le sumo 2 días injustificados que se le descontaron</t>
+  </si>
+  <si>
+    <t>Estaba en Recoleta en el original x error</t>
   </si>
 </sst>
 </file>
@@ -630,28 +633,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P314"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="4"/>
-    <col min="2" max="2" width="9.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5546875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="10.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" style="4"/>
+    <col min="2" max="2" width="9.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.90625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.54296875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="10.453125" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" style="4" customWidth="1"/>
-    <col min="11" max="11" width="6.44140625" style="4" customWidth="1"/>
-    <col min="12" max="12" width="13.109375" style="4" customWidth="1"/>
-    <col min="13" max="13" width="7.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.44140625" style="4" customWidth="1"/>
-    <col min="15" max="15" width="6.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="11.5546875" style="4"/>
+    <col min="9" max="9" width="11.453125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" style="4" customWidth="1"/>
+    <col min="11" max="11" width="6.453125" style="4" customWidth="1"/>
+    <col min="12" max="12" width="13.08984375" style="4" customWidth="1"/>
+    <col min="13" max="13" width="7.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.453125" style="4" customWidth="1"/>
+    <col min="15" max="15" width="6.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.08984375" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="11.54296875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -701,7 +704,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>45901</v>
       </c>
@@ -719,7 +722,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>45901</v>
       </c>
@@ -737,7 +740,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>45901</v>
       </c>
@@ -755,7 +758,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>45901</v>
       </c>
@@ -770,7 +773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>45901</v>
       </c>
@@ -785,7 +788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>45901</v>
       </c>
@@ -803,7 +806,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>45901</v>
       </c>
@@ -821,7 +824,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>45901</v>
       </c>
@@ -842,7 +845,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>45901</v>
       </c>
@@ -863,7 +866,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>45901</v>
       </c>
@@ -885,7 +888,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>45901</v>
       </c>
@@ -903,7 +906,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>45901</v>
       </c>
@@ -918,7 +921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>45901</v>
       </c>
@@ -939,7 +942,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>45901</v>
       </c>
@@ -960,7 +963,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>45901</v>
       </c>
@@ -978,7 +981,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>45901</v>
       </c>
@@ -996,7 +999,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>45901</v>
       </c>
@@ -1011,7 +1014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>45901</v>
       </c>
@@ -1029,7 +1032,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>45901</v>
       </c>
@@ -1050,7 +1053,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>45901</v>
       </c>
@@ -1068,7 +1071,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>45901</v>
       </c>
@@ -1089,7 +1092,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>45901</v>
       </c>
@@ -1107,7 +1110,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>45901</v>
       </c>
@@ -1128,7 +1131,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>45901</v>
       </c>
@@ -1146,7 +1149,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>45931</v>
       </c>
@@ -1167,7 +1170,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>45931</v>
       </c>
@@ -1188,7 +1191,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>45931</v>
       </c>
@@ -1206,7 +1209,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>45931</v>
       </c>
@@ -1221,7 +1224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>45931</v>
       </c>
@@ -1239,7 +1242,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>45931</v>
       </c>
@@ -1257,7 +1260,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>45931</v>
       </c>
@@ -1275,7 +1278,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>45931</v>
       </c>
@@ -1299,7 +1302,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>45931</v>
       </c>
@@ -1317,7 +1320,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>45931</v>
       </c>
@@ -1335,7 +1338,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>45931</v>
       </c>
@@ -1356,7 +1359,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>45931</v>
       </c>
@@ -1377,7 +1380,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>45931</v>
       </c>
@@ -1395,7 +1398,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>45931</v>
       </c>
@@ -1416,7 +1419,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>45931</v>
       </c>
@@ -1434,7 +1437,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>45931</v>
       </c>
@@ -1455,7 +1458,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>45931</v>
       </c>
@@ -1476,7 +1479,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>45931</v>
       </c>
@@ -1499,7 +1502,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>45931</v>
       </c>
@@ -1517,7 +1520,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>45931</v>
       </c>
@@ -1535,7 +1538,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A46" s="3">
         <v>45931</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A47" s="3">
         <v>45931</v>
       </c>
@@ -1571,7 +1574,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A48" s="3">
         <v>45931</v>
       </c>
@@ -1589,7 +1592,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A49" s="3">
         <v>45931</v>
       </c>
@@ -1607,7 +1610,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A50" s="3">
         <v>45931</v>
       </c>
@@ -1625,7 +1628,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A51" s="3">
         <v>45931</v>
       </c>
@@ -1644,7 +1647,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A52" s="3">
         <v>45931</v>
       </c>
@@ -1662,7 +1665,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A53" s="3">
         <v>45962</v>
       </c>
@@ -1687,7 +1690,7 @@
       </c>
       <c r="P53" s="6"/>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A54" s="3">
         <v>45962</v>
       </c>
@@ -1705,7 +1708,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A55" s="3">
         <v>45962</v>
       </c>
@@ -1723,7 +1726,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A56" s="3">
         <v>45962</v>
       </c>
@@ -1738,7 +1741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A57" s="3">
         <v>45962</v>
       </c>
@@ -1756,7 +1759,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A58" s="3">
         <v>45962</v>
       </c>
@@ -1774,7 +1777,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A59" s="3">
         <v>45962</v>
       </c>
@@ -1792,7 +1795,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A60" s="3">
         <v>45962</v>
       </c>
@@ -1813,7 +1816,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A61" s="3">
         <v>45962</v>
       </c>
@@ -1831,7 +1834,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A62" s="3">
         <v>45962</v>
       </c>
@@ -1849,7 +1852,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A63" s="3">
         <v>45962</v>
       </c>
@@ -1870,7 +1873,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A64" s="3">
         <v>45962</v>
       </c>
@@ -1888,7 +1891,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A65" s="3">
         <v>45962</v>
       </c>
@@ -1909,7 +1912,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A66" s="3">
         <v>45962</v>
       </c>
@@ -1927,7 +1930,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A67" s="3">
         <v>45962</v>
       </c>
@@ -1945,7 +1948,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A68" s="3">
         <v>45962</v>
       </c>
@@ -1969,7 +1972,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A69" s="3">
         <v>45962</v>
       </c>
@@ -1990,7 +1993,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A70" s="3">
         <v>45962</v>
       </c>
@@ -2011,7 +2014,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A71" s="3">
         <v>45962</v>
       </c>
@@ -2029,7 +2032,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A72" s="3">
         <v>45962</v>
       </c>
@@ -2047,7 +2050,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A73" s="3">
         <v>45962</v>
       </c>
@@ -2068,7 +2071,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A74" s="3">
         <v>45962</v>
       </c>
@@ -2086,7 +2089,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A75" s="3">
         <v>45962</v>
       </c>
@@ -2104,7 +2107,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A76" s="3">
         <v>45962</v>
       </c>
@@ -2122,7 +2125,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="77" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A77" s="3">
         <v>45962</v>
       </c>
@@ -2143,7 +2146,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A78" s="3">
         <v>45962</v>
       </c>
@@ -2161,7 +2164,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A79" s="3">
         <v>45962</v>
       </c>
@@ -2179,7 +2182,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A80" s="3">
         <v>45962</v>
       </c>
@@ -2200,7 +2203,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A81" s="3">
         <v>45962</v>
       </c>
@@ -2221,7 +2224,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A82" s="3">
         <v>45962</v>
       </c>
@@ -2239,7 +2242,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A83" s="3">
         <v>45992</v>
       </c>
@@ -2261,7 +2264,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A84" s="3">
         <v>45992</v>
       </c>
@@ -2283,7 +2286,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A85" s="3">
         <v>45992</v>
       </c>
@@ -2301,7 +2304,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A86" s="3">
         <v>45992</v>
       </c>
@@ -2319,7 +2322,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A87" s="3">
         <v>45992</v>
       </c>
@@ -2337,7 +2340,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A88" s="3">
         <v>45992</v>
       </c>
@@ -2355,7 +2358,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A89" s="3">
         <v>45992</v>
       </c>
@@ -2373,7 +2376,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A90" s="3">
         <v>45992</v>
       </c>
@@ -2391,7 +2394,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A91" s="3">
         <v>45992</v>
       </c>
@@ -2409,7 +2412,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A92" s="3">
         <v>45992</v>
       </c>
@@ -2427,7 +2430,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A93" s="3">
         <v>45992</v>
       </c>
@@ -2448,7 +2451,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A94" s="3">
         <v>45992</v>
       </c>
@@ -2470,7 +2473,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A95" s="3">
         <v>45992</v>
       </c>
@@ -2492,7 +2495,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A96" s="3">
         <v>45992</v>
       </c>
@@ -2514,7 +2517,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A97" s="3">
         <v>45992</v>
       </c>
@@ -2535,7 +2538,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A98" s="3">
         <v>45992</v>
       </c>
@@ -2557,7 +2560,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A99" s="3">
         <v>45992</v>
       </c>
@@ -2582,7 +2585,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A100" s="3">
         <v>45992</v>
       </c>
@@ -2600,7 +2603,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A101" s="3">
         <v>45992</v>
       </c>
@@ -2618,7 +2621,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A102" s="3">
         <v>45992</v>
       </c>
@@ -2636,7 +2639,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A103" s="3">
         <v>45992</v>
       </c>
@@ -2654,7 +2657,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A104" s="3">
         <v>45992</v>
       </c>
@@ -2672,7 +2675,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A105" s="3">
         <v>45992</v>
       </c>
@@ -2690,7 +2693,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A106" s="3">
         <v>45992</v>
       </c>
@@ -2708,7 +2711,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A107" s="3">
         <v>45992</v>
       </c>
@@ -2726,7 +2729,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A108" s="3">
         <v>45992</v>
       </c>
@@ -2744,7 +2747,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A109" s="3">
         <v>45992</v>
       </c>
@@ -2762,7 +2765,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A110" s="3">
         <v>45992</v>
       </c>
@@ -2780,7 +2783,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A111" s="3">
         <v>45992</v>
       </c>
@@ -2798,7 +2801,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A112" s="3">
         <v>45992</v>
       </c>
@@ -2816,7 +2819,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A113" s="3">
         <v>45992</v>
       </c>
@@ -2834,7 +2837,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A114" s="3">
         <v>45992</v>
       </c>
@@ -2852,7 +2855,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A115" s="3">
         <v>46023</v>
       </c>
@@ -2873,7 +2876,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A116" s="3">
         <v>46023</v>
       </c>
@@ -2891,7 +2894,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A117" s="3">
         <v>46023</v>
       </c>
@@ -2912,7 +2915,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A118" s="3">
         <v>46023</v>
       </c>
@@ -2930,7 +2933,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A119" s="3">
         <v>46023</v>
       </c>
@@ -2951,7 +2954,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A120" s="3">
         <v>46023</v>
       </c>
@@ -2969,7 +2972,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A121" s="3">
         <v>46023</v>
       </c>
@@ -2987,7 +2990,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A122" s="3">
         <v>46023</v>
       </c>
@@ -3005,7 +3008,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A123" s="3">
         <v>46023</v>
       </c>
@@ -3026,7 +3029,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A124" s="3">
         <v>46023</v>
       </c>
@@ -3044,7 +3047,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A125" s="3">
         <v>46023</v>
       </c>
@@ -3062,7 +3065,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A126" s="3">
         <v>46023</v>
       </c>
@@ -3080,7 +3083,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A127" s="3">
         <v>46023</v>
       </c>
@@ -3098,7 +3101,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A128" s="3">
         <v>46023</v>
       </c>
@@ -3120,7 +3123,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A129" s="3">
         <v>46023</v>
       </c>
@@ -3138,7 +3141,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A130" s="3">
         <v>46023</v>
       </c>
@@ -3156,7 +3159,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A131" s="3">
         <v>46023</v>
       </c>
@@ -3173,7 +3176,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A132" s="3">
         <v>46023</v>
       </c>
@@ -3194,7 +3197,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A133" s="3">
         <v>46023</v>
       </c>
@@ -3218,7 +3221,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A134" s="3">
         <v>46023</v>
       </c>
@@ -3240,7 +3243,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A135" s="3">
         <v>46023</v>
       </c>
@@ -3261,7 +3264,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A136" s="3">
         <v>46023</v>
       </c>
@@ -3285,7 +3288,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A137" s="3">
         <v>46023</v>
       </c>
@@ -3303,7 +3306,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A138" s="3">
         <v>46023</v>
       </c>
@@ -3327,7 +3330,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A139" s="3">
         <v>46023</v>
       </c>
@@ -3345,7 +3348,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A140" s="3">
         <v>46023</v>
       </c>
@@ -3363,7 +3366,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A141" s="3">
         <v>46023</v>
       </c>
@@ -3384,7 +3387,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A142" s="3">
         <v>46023</v>
       </c>
@@ -3402,7 +3405,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A143" s="3">
         <v>46023</v>
       </c>
@@ -3420,7 +3423,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A144" s="3">
         <v>46023</v>
       </c>
@@ -3438,7 +3441,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A145" s="3">
         <v>46023</v>
       </c>
@@ -3456,7 +3459,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A146" s="3">
         <v>46023</v>
       </c>
@@ -3477,7 +3480,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="147" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A147" s="3">
         <v>46023</v>
       </c>
@@ -3498,7 +3501,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="148" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A148" s="3">
         <v>46054</v>
       </c>
@@ -3522,7 +3525,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A149" s="3">
         <v>46054</v>
       </c>
@@ -3540,7 +3543,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A150" s="3">
         <v>46054</v>
       </c>
@@ -3558,7 +3561,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A151" s="3">
         <v>46054</v>
       </c>
@@ -3579,7 +3582,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A152" s="3">
         <v>46054</v>
       </c>
@@ -3597,7 +3600,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="153" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A153" s="3">
         <v>46054</v>
       </c>
@@ -3615,7 +3618,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A154" s="3">
         <v>46054</v>
       </c>
@@ -3636,7 +3639,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="155" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A155" s="3">
         <v>46054</v>
       </c>
@@ -3654,7 +3657,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A156" s="3">
         <v>46054</v>
       </c>
@@ -3675,7 +3678,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="157" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A157" s="3">
         <v>46054</v>
       </c>
@@ -3699,7 +3702,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="158" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A158" s="3">
         <v>46054</v>
       </c>
@@ -3717,7 +3720,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A159" s="3">
         <v>46054</v>
       </c>
@@ -3735,7 +3738,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A160" s="3">
         <v>46054</v>
       </c>
@@ -3757,7 +3760,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="161" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A161" s="3">
         <v>46054</v>
       </c>
@@ -3775,7 +3778,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="162" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A162" s="3">
         <v>46054</v>
       </c>
@@ -3796,7 +3799,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="163" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A163" s="3">
         <v>46054</v>
       </c>
@@ -3814,7 +3817,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A164" s="3">
         <v>46054</v>
       </c>
@@ -3832,7 +3835,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="165" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A165" s="3">
         <v>46054</v>
       </c>
@@ -3850,7 +3853,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="166" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A166" s="3">
         <v>46054</v>
       </c>
@@ -3871,7 +3874,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A167" s="3">
         <v>46054</v>
       </c>
@@ -3898,7 +3901,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A168" s="3">
         <v>46054</v>
       </c>
@@ -3919,7 +3922,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A169" s="3">
         <v>46054</v>
       </c>
@@ -3940,7 +3943,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A170" s="3">
         <v>46054</v>
       </c>
@@ -3958,7 +3961,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="171" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A171" s="3">
         <v>46054</v>
       </c>
@@ -3976,7 +3979,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="172" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A172" s="3">
         <v>46054</v>
       </c>
@@ -3997,7 +4000,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A173" s="3">
         <v>46054</v>
       </c>
@@ -4015,7 +4018,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="174" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A174" s="3">
         <v>46054</v>
       </c>
@@ -4036,7 +4039,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A175" s="3">
         <v>46054</v>
       </c>
@@ -4054,7 +4057,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="176" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A176" s="3">
         <v>46054</v>
       </c>
@@ -4075,7 +4078,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A177" s="3">
         <v>46054</v>
       </c>
@@ -4093,7 +4096,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A178" s="3">
         <v>46054</v>
       </c>
@@ -4117,7 +4120,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A179" s="3">
         <v>46082</v>
       </c>
@@ -4138,7 +4141,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A180" s="3">
         <v>46082</v>
       </c>
@@ -4156,7 +4159,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A181" s="3">
         <v>46082</v>
       </c>
@@ -4174,7 +4177,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A182" s="3">
         <v>46082</v>
       </c>
@@ -4192,7 +4195,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A183" s="3">
         <v>46082</v>
       </c>
@@ -4210,7 +4213,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A184" s="3">
         <v>46082</v>
       </c>
@@ -4231,7 +4234,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A185" s="3">
         <v>46082</v>
       </c>
@@ -4249,7 +4252,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A186" s="3">
         <v>46082</v>
       </c>
@@ -4270,7 +4273,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A187" s="3">
         <v>46082</v>
       </c>
@@ -4288,7 +4291,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A188" s="3">
         <v>46082</v>
       </c>
@@ -4309,7 +4312,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A189" s="3">
         <v>46082</v>
       </c>
@@ -4330,7 +4333,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A190" s="3">
         <v>46082</v>
       </c>
@@ -4348,7 +4351,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A191" s="3">
         <v>46082</v>
       </c>
@@ -4366,7 +4369,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A192" s="3">
         <v>46082</v>
       </c>
@@ -4384,7 +4387,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A193" s="3">
         <v>46082</v>
       </c>
@@ -4405,7 +4408,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A194" s="3">
         <v>46082</v>
       </c>
@@ -4426,7 +4429,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A195" s="3">
         <v>46082</v>
       </c>
@@ -4447,7 +4450,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A196" s="3">
         <v>46082</v>
       </c>
@@ -4471,7 +4474,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A197" s="3">
         <v>46082</v>
       </c>
@@ -4492,7 +4495,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A198" s="3">
         <v>46082</v>
       </c>
@@ -4513,7 +4516,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A199" s="3">
         <v>46082</v>
       </c>
@@ -4531,7 +4534,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A200" s="3">
         <v>46082</v>
       </c>
@@ -4552,7 +4555,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A201" s="3">
         <v>46082</v>
       </c>
@@ -4570,7 +4573,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A202" s="3">
         <v>46082</v>
       </c>
@@ -4591,7 +4594,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="203" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A203" s="3">
         <v>46082</v>
       </c>
@@ -4609,7 +4612,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="204" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A204" s="3">
         <v>46082</v>
       </c>
@@ -4630,7 +4633,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="205" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A205" s="3">
         <v>46082</v>
       </c>
@@ -4648,7 +4651,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A206" s="3">
         <v>46082</v>
       </c>
@@ -4669,7 +4672,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A207" s="3">
         <v>46113</v>
       </c>
@@ -4690,7 +4693,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A208" s="3">
         <v>46113</v>
       </c>
@@ -4708,7 +4711,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A209" s="3">
         <v>46113</v>
       </c>
@@ -4726,7 +4729,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A210" s="3">
         <v>46113</v>
       </c>
@@ -4744,7 +4747,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A211" s="3">
         <v>46113</v>
       </c>
@@ -4762,7 +4765,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="212" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A212" s="3">
         <v>46113</v>
       </c>
@@ -4783,7 +4786,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="213" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A213" s="3">
         <v>46113</v>
       </c>
@@ -4801,7 +4804,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="214" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A214" s="3">
         <v>46113</v>
       </c>
@@ -4819,7 +4822,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="215" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A215" s="3">
         <v>46113</v>
       </c>
@@ -4840,7 +4843,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="216" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A216" s="3">
         <v>46113</v>
       </c>
@@ -4858,7 +4861,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="217" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A217" s="3">
         <v>46113</v>
       </c>
@@ -4876,7 +4879,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="218" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A218" s="3">
         <v>46113</v>
       </c>
@@ -4894,7 +4897,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="219" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A219" s="3">
         <v>46113</v>
       </c>
@@ -4915,7 +4918,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="220" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A220" s="3">
         <v>46113</v>
       </c>
@@ -4936,7 +4939,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="221" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A221" s="3">
         <v>46113</v>
       </c>
@@ -4954,7 +4957,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="222" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A222" s="3">
         <v>46113</v>
       </c>
@@ -4972,7 +4975,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="223" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A223" s="3">
         <v>46113</v>
       </c>
@@ -4990,7 +4993,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="224" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A224" s="3">
         <v>46113</v>
       </c>
@@ -5008,7 +5011,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="225" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A225" s="3">
         <v>46113</v>
       </c>
@@ -5026,7 +5029,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="226" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A226" s="3">
         <v>46113</v>
       </c>
@@ -5047,7 +5050,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="227" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A227" s="3">
         <v>46113</v>
       </c>
@@ -5065,7 +5068,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="228" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A228" s="3">
         <v>46113</v>
       </c>
@@ -5086,7 +5089,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="229" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A229" s="3">
         <v>46113</v>
       </c>
@@ -5104,7 +5107,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="230" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A230" s="3">
         <v>46113</v>
       </c>
@@ -5122,7 +5125,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="231" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A231" s="3">
         <v>46113</v>
       </c>
@@ -5140,7 +5143,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="232" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A232" s="3">
         <v>46113</v>
       </c>
@@ -5161,7 +5164,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="233" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A233" s="3">
         <v>46113</v>
       </c>
@@ -5179,7 +5182,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="234" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A234" s="3">
         <v>46113</v>
       </c>
@@ -5197,7 +5200,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="235" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A235" s="3">
         <v>46143</v>
       </c>
@@ -5218,7 +5221,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="236" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A236" s="3">
         <v>46143</v>
       </c>
@@ -5236,7 +5239,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="237" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A237" s="3">
         <v>46143</v>
       </c>
@@ -5254,7 +5257,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="238" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A238" s="3">
         <v>46143</v>
       </c>
@@ -5272,7 +5275,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="239" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A239" s="3">
         <v>46143</v>
       </c>
@@ -5290,7 +5293,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="240" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A240" s="3">
         <v>46143</v>
       </c>
@@ -5308,7 +5311,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="241" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A241" s="3">
         <v>46143</v>
       </c>
@@ -5326,7 +5329,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="242" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A242" s="3">
         <v>46143</v>
       </c>
@@ -5350,7 +5353,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="243" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A243" s="3">
         <v>46143</v>
       </c>
@@ -5368,7 +5371,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="244" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A244" s="3">
         <v>46143</v>
       </c>
@@ -5386,7 +5389,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="245" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A245" s="3">
         <v>46143</v>
       </c>
@@ -5404,7 +5407,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="246" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A246" s="3">
         <v>46143</v>
       </c>
@@ -5422,7 +5425,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="247" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A247" s="3">
         <v>46143</v>
       </c>
@@ -5443,7 +5446,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="248" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A248" s="3">
         <v>46143</v>
       </c>
@@ -5461,7 +5464,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="249" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A249" s="3">
         <v>46143</v>
       </c>
@@ -5482,7 +5485,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="250" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A250" s="3">
         <v>46143</v>
       </c>
@@ -5503,7 +5506,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="251" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A251" s="3">
         <v>46143</v>
       </c>
@@ -5524,7 +5527,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="252" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A252" s="3">
         <v>46143</v>
       </c>
@@ -5542,7 +5545,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="253" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A253" s="3">
         <v>46143</v>
       </c>
@@ -5560,7 +5563,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="254" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A254" s="3">
         <v>46143</v>
       </c>
@@ -5581,7 +5584,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="255" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A255" s="3">
         <v>46143</v>
       </c>
@@ -5599,7 +5602,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="256" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A256" s="3">
         <v>46143</v>
       </c>
@@ -5617,7 +5620,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="257" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A257" s="3">
         <v>46143</v>
       </c>
@@ -5641,7 +5644,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="258" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A258" s="3">
         <v>46143</v>
       </c>
@@ -5659,7 +5662,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="259" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A259" s="3">
         <v>46143</v>
       </c>
@@ -5680,7 +5683,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="260" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A260" s="3">
         <v>46143</v>
       </c>
@@ -5701,7 +5704,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="261" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A261" s="3">
         <v>46143</v>
       </c>
@@ -5719,7 +5722,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="262" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A262" s="3">
         <v>46174</v>
       </c>
@@ -5729,15 +5732,18 @@
       <c r="C262" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H262" s="4">
+      <c r="D262" s="5">
         <v>123</v>
       </c>
       <c r="O262" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(D262:N262)</f>
         <v>123</v>
       </c>
-    </row>
-    <row r="263" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P262" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="263" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A263" s="3">
         <v>46174</v>
       </c>
@@ -5755,7 +5761,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="264" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A264" s="3">
         <v>46174</v>
       </c>
@@ -5773,7 +5779,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="265" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A265" s="3">
         <v>46174</v>
       </c>
@@ -5791,7 +5797,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="266" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A266" s="3">
         <v>46174</v>
       </c>
@@ -5809,7 +5815,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="267" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A267" s="3">
         <v>46174</v>
       </c>
@@ -5830,7 +5836,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="268" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A268" s="3">
         <v>46174</v>
       </c>
@@ -5848,7 +5854,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="269" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A269" s="3">
         <v>46174</v>
       </c>
@@ -5869,7 +5875,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="270" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A270" s="3">
         <v>46174</v>
       </c>
@@ -5887,7 +5893,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="271" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A271" s="3">
         <v>46174</v>
       </c>
@@ -5905,7 +5911,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="272" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A272" s="3">
         <v>46174</v>
       </c>
@@ -5923,7 +5929,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="273" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A273" s="3">
         <v>46174</v>
       </c>
@@ -5941,7 +5947,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="274" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A274" s="3">
         <v>46174</v>
       </c>
@@ -5962,7 +5968,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="275" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A275" s="3">
         <v>46174</v>
       </c>
@@ -5980,7 +5986,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="276" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A276" s="3">
         <v>46174</v>
       </c>
@@ -6001,7 +6007,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="277" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A277" s="3">
         <v>46174</v>
       </c>
@@ -6022,7 +6028,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="278" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A278" s="3">
         <v>46174</v>
       </c>
@@ -6040,7 +6046,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="279" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A279" s="3">
         <v>46174</v>
       </c>
@@ -6058,7 +6064,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="280" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A280" s="3">
         <v>46174</v>
       </c>
@@ -6076,7 +6082,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="281" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A281" s="3">
         <v>46174</v>
       </c>
@@ -6094,7 +6100,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="282" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A282" s="3">
         <v>46174</v>
       </c>
@@ -6115,7 +6121,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="283" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A283" s="3">
         <v>46174</v>
       </c>
@@ -6133,7 +6139,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="284" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A284" s="3">
         <v>46174</v>
       </c>
@@ -6154,7 +6160,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="285" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A285" s="3">
         <v>46174</v>
       </c>
@@ -6175,7 +6181,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="286" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A286" s="3">
         <v>46174</v>
       </c>
@@ -6193,7 +6199,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="287" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A287" s="3">
         <v>46174</v>
       </c>
@@ -6214,7 +6220,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="288" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A288" s="3">
         <v>46174</v>
       </c>
@@ -6232,7 +6238,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="289" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A289" s="3">
         <v>46204</v>
       </c>
@@ -6250,7 +6256,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="290" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A290" s="3">
         <v>46204</v>
       </c>
@@ -6268,7 +6274,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="291" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A291" s="3">
         <v>46204</v>
       </c>
@@ -6286,7 +6292,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="292" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A292" s="3">
         <v>46204</v>
       </c>
@@ -6304,7 +6310,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="293" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A293" s="3">
         <v>46204</v>
       </c>
@@ -6322,7 +6328,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="294" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A294" s="3">
         <v>46204</v>
       </c>
@@ -6346,7 +6352,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="295" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A295" s="3">
         <v>46204</v>
       </c>
@@ -6364,7 +6370,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="296" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A296" s="3">
         <v>46204</v>
       </c>
@@ -6385,7 +6391,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="297" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A297" s="3">
         <v>46204</v>
       </c>
@@ -6406,7 +6412,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="298" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A298" s="3">
         <v>46204</v>
       </c>
@@ -6424,7 +6430,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="299" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A299" s="3">
         <v>46204</v>
       </c>
@@ -6445,7 +6451,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="300" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A300" s="3">
         <v>46204</v>
       </c>
@@ -6463,7 +6469,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="301" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A301" s="3">
         <v>46204</v>
       </c>
@@ -6484,7 +6490,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="302" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A302" s="3">
         <v>46204</v>
       </c>
@@ -6502,7 +6508,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="303" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A303" s="3">
         <v>46204</v>
       </c>
@@ -6523,7 +6529,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="304" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A304" s="3">
         <v>46204</v>
       </c>
@@ -6544,7 +6550,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="305" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A305" s="3">
         <v>46204</v>
       </c>
@@ -6562,7 +6568,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="306" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A306" s="3">
         <v>46204</v>
       </c>
@@ -6580,7 +6586,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="307" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A307" s="3">
         <v>46204</v>
       </c>
@@ -6598,7 +6604,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="308" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A308" s="3">
         <v>46204</v>
       </c>
@@ -6616,7 +6622,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="309" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A309" s="3">
         <v>46204</v>
       </c>
@@ -6637,7 +6643,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="310" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A310" s="3">
         <v>46204</v>
       </c>
@@ -6655,7 +6661,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="311" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A311" s="3">
         <v>46204</v>
       </c>
@@ -6673,7 +6679,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="312" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A312" s="3">
         <v>46204</v>
       </c>
@@ -6694,7 +6700,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="313" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A313" s="3">
         <v>46204</v>
       </c>
@@ -6712,7 +6718,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="314" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A314" s="3">
         <v>46204</v>
       </c>
@@ -6734,7 +6740,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O288"/>
+  <autoFilter ref="A1:O315"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6742,12 +6748,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F41"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -6767,7 +6773,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -6781,7 +6787,7 @@
         <v>46088</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>3</v>
       </c>
@@ -6791,8 +6797,14 @@
       <c r="C3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E3" s="8">
+        <v>46174</v>
+      </c>
+      <c r="F3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>4</v>
       </c>
@@ -6803,7 +6815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>10</v>
       </c>
@@ -6814,7 +6826,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>11</v>
       </c>
@@ -6825,7 +6837,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>12</v>
       </c>
@@ -6836,7 +6848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>13</v>
       </c>
@@ -6850,7 +6862,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>14</v>
       </c>
@@ -6861,7 +6873,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>15</v>
       </c>
@@ -6872,7 +6884,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>18</v>
       </c>
@@ -6883,7 +6895,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>19</v>
       </c>
@@ -6894,7 +6906,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>20</v>
       </c>
@@ -6905,7 +6917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <v>21</v>
       </c>
@@ -6919,7 +6931,7 @@
         <v>46034</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <v>27</v>
       </c>
@@ -6930,7 +6942,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <v>28</v>
       </c>
@@ -6941,7 +6953,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>29</v>
       </c>
@@ -6959,7 +6971,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>30</v>
       </c>
@@ -6973,7 +6985,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>31</v>
       </c>
@@ -6984,7 +6996,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>32</v>
       </c>
@@ -6998,7 +7010,7 @@
         <v>46076</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>34</v>
       </c>
@@ -7012,7 +7024,7 @@
         <v>45998</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
         <v>36</v>
       </c>
@@ -7023,7 +7035,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
         <v>38</v>
       </c>
@@ -7037,7 +7049,7 @@
         <v>46123</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
         <v>39</v>
       </c>
@@ -7055,7 +7067,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
         <v>40</v>
       </c>
@@ -7069,7 +7081,7 @@
         <v>46123</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
         <v>41</v>
       </c>
@@ -7086,7 +7098,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="4">
         <v>42</v>
       </c>
@@ -7097,7 +7109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>43</v>
       </c>
@@ -7111,7 +7123,7 @@
         <v>46007</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="4">
         <v>44</v>
       </c>
@@ -7131,7 +7143,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="4">
         <v>45</v>
       </c>
@@ -7145,7 +7157,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="4">
         <v>46</v>
       </c>
@@ -7159,7 +7171,7 @@
         <v>46097</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="4">
         <v>47</v>
       </c>
@@ -7173,7 +7185,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="4">
         <v>49</v>
       </c>
@@ -7184,7 +7196,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>51</v>
       </c>
@@ -7198,7 +7210,7 @@
         <v>46032</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="4">
         <v>52</v>
       </c>
@@ -7209,7 +7221,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="4">
         <v>53</v>
       </c>
@@ -7223,7 +7235,7 @@
         <v>46076</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="4">
         <v>54</v>
       </c>
@@ -7234,7 +7246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="4">
         <v>55</v>
       </c>
@@ -7248,7 +7260,7 @@
         <v>46119</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="4">
         <v>58</v>
       </c>
@@ -7260,7 +7272,7 @@
       </c>
       <c r="D39" s="8"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="4">
         <v>59</v>
       </c>
@@ -7274,7 +7286,7 @@
         <v>46209</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="4">
         <v>63</v>
       </c>

</xml_diff>

<commit_message>
sin venta joyería. Creé R para automatizar tabla horas de vendedoras por mes. Empecé a buscar archivos para obtener datos de clientes
</commit_message>
<xml_diff>
--- a/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
+++ b/Reporte_gastos/Sueldos/Horas trabajadas Tiendas desde 2025-09.xlsx
@@ -9,11 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6310"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6310" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="tabla x hora" sheetId="1" r:id="rId1"/>
     <sheet name="vendedora-tienda" sheetId="3" r:id="rId2"/>
+    <sheet name="alias" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tabla x hora'!$A$1:$O$315</definedName>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="97">
   <si>
     <t>Florida</t>
   </si>
@@ -257,6 +258,69 @@
   </si>
   <si>
     <t>Estaba en Recoleta en el original x error</t>
+  </si>
+  <si>
+    <t>Sin identificar (10-2025, El Solar, 41 hs)</t>
+  </si>
+  <si>
+    <t>Ronald Julieta</t>
+  </si>
+  <si>
+    <t>Hernandez Guerrero Helen</t>
+  </si>
+  <si>
+    <t>Ariganiello Melina</t>
+  </si>
+  <si>
+    <t>Arguello Melina</t>
+  </si>
+  <si>
+    <t>Noelia Gomez Ayala</t>
+  </si>
+  <si>
+    <t>Gil Matquez Johana</t>
+  </si>
+  <si>
+    <t>Gil Marquwz Johana</t>
+  </si>
+  <si>
+    <t>Gil Marquez Johana</t>
+  </si>
+  <si>
+    <t>Sayarly Choque</t>
+  </si>
+  <si>
+    <t>Bogaron gomez Noelia</t>
+  </si>
+  <si>
+    <t>Cardozo Trinidad</t>
+  </si>
+  <si>
+    <t>Ochoa Duran Talia</t>
+  </si>
+  <si>
+    <t>Giordano Carolina</t>
+  </si>
+  <si>
+    <t>Giordano Caroline</t>
+  </si>
+  <si>
+    <t>Bonino Gisella</t>
+  </si>
+  <si>
+    <t>Baragatti Anabela</t>
+  </si>
+  <si>
+    <t>De Brito</t>
+  </si>
+  <si>
+    <t>Comentario</t>
+  </si>
+  <si>
+    <t>Nombre_canonico</t>
+  </si>
+  <si>
+    <t>Nombre_premios</t>
   </si>
 </sst>
 </file>
@@ -267,7 +331,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -295,6 +359,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -324,7 +394,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -340,6 +410,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -7310,4 +7381,218 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="4" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9">
+        <v>45</v>
+      </c>
+      <c r="C9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11">
+        <v>49</v>
+      </c>
+      <c r="C11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13">
+        <v>49</v>
+      </c>
+      <c r="C13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15">
+        <v>59</v>
+      </c>
+      <c r="C15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16">
+        <v>59</v>
+      </c>
+      <c r="C16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17">
+        <v>60</v>
+      </c>
+      <c r="C17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>